<commit_message>
more of the penultimate update
</commit_message>
<xml_diff>
--- a/intermediate/dashboard_output_gender.xlsx
+++ b/intermediate/dashboard_output_gender.xlsx
@@ -457,13 +457,13 @@
         </is>
       </c>
       <c r="H2">
-        <v>-37.30555555555582</v>
+        <v>-36.80769233684551</v>
       </c>
       <c r="I2">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="J2">
-        <v>6.5</v>
+        <v>2.6</v>
       </c>
       <c r="K2">
         <v>53.3</v>
@@ -482,7 +482,7 @@
         <v>2015</v>
       </c>
       <c r="O2">
-        <v>55.7</v>
+        <v>56.05588235294112</v>
       </c>
     </row>
     <row r="3">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="H3">
-        <v>1.6875</v>
+        <v>1.875658004914925</v>
       </c>
       <c r="I3">
         <v>2023</v>
@@ -536,7 +536,7 @@
         <v>2015</v>
       </c>
       <c r="O3">
-        <v>73.10000000000001</v>
+        <v>72.87815078236147</v>
       </c>
     </row>
     <row r="4">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="H4">
-        <v>4.499999999999964</v>
+        <v>7.67750368611437</v>
       </c>
       <c r="I4">
         <v>2023</v>
@@ -590,7 +590,7 @@
         <v>2015</v>
       </c>
       <c r="O4">
-        <v>85.20000000000005</v>
+        <v>84.51233574131409</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="H5">
-        <v>4.572916666666689</v>
+        <v>5.470000115780927</v>
       </c>
       <c r="I5">
         <v>2023</v>
@@ -644,7 +644,7 @@
         <v>2015</v>
       </c>
       <c r="O5">
-        <v>46.36666666666661</v>
+        <v>46.06896551724144</v>
       </c>
     </row>
     <row r="6">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="H6">
-        <v>1.062499999999993</v>
+        <v>1.501528496013805</v>
       </c>
       <c r="I6">
         <v>2023</v>
@@ -698,7 +698,7 @@
         <v>2015</v>
       </c>
       <c r="O6">
-        <v>86</v>
+        <v>85.54598039215685</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="H7">
-        <v>6.489583333333179</v>
+        <v>9.850563668826972</v>
       </c>
       <c r="I7">
         <v>2023</v>
@@ -752,7 +752,7 @@
         <v>2015</v>
       </c>
       <c r="O7">
-        <v>78.17500000000003</v>
+        <v>77.52371700879768</v>
       </c>
     </row>
     <row r="8">
@@ -780,12 +780,18 @@
           <t>AUS</t>
         </is>
       </c>
+      <c r="H8">
+        <v>-9.166666666666657</v>
+      </c>
       <c r="I8">
         <v>2023</v>
       </c>
       <c r="J8">
         <v>91.7</v>
       </c>
+      <c r="K8">
+        <v>93.60000000000001</v>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>45.0.0</t>
@@ -795,6 +801,12 @@
         <is>
           <t>Women political empowerment index</t>
         </is>
+      </c>
+      <c r="N8">
+        <v>2015</v>
+      </c>
+      <c r="O8">
+        <v>93.68000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -890,7 +902,7 @@
         <v>2015</v>
       </c>
       <c r="O10">
-        <v>69.2</v>
+        <v>69.15499999999989</v>
       </c>
     </row>
     <row r="11">
@@ -919,7 +931,7 @@
         </is>
       </c>
       <c r="H11">
-        <v>2.59375</v>
+        <v>2.645748987854283</v>
       </c>
       <c r="I11">
         <v>2023</v>
@@ -944,7 +956,7 @@
         <v>2015</v>
       </c>
       <c r="O11">
-        <v>62.7</v>
+        <v>62.57526315789475</v>
       </c>
     </row>
     <row r="12">
@@ -1015,7 +1027,7 @@
         </is>
       </c>
       <c r="H13">
-        <v>2.41666666666665</v>
+        <v>3.86207970950619</v>
       </c>
       <c r="I13">
         <v>2023</v>
@@ -1040,7 +1052,7 @@
         <v>2015</v>
       </c>
       <c r="O13">
-        <v>85.73333333333335</v>
+        <v>85.19632352941177</v>
       </c>
     </row>
     <row r="14">
@@ -1069,7 +1081,7 @@
         </is>
       </c>
       <c r="H14">
-        <v>-1.78125</v>
+        <v>-1.89182437208752</v>
       </c>
       <c r="I14">
         <v>2023</v>
@@ -1094,7 +1106,7 @@
         <v>2015</v>
       </c>
       <c r="O14">
-        <v>76.7</v>
+        <v>76.18827094474153</v>
       </c>
     </row>
     <row r="15">
@@ -1123,7 +1135,7 @@
         </is>
       </c>
       <c r="H15">
-        <v>-0.125</v>
+        <v>-0.1282051282051384</v>
       </c>
       <c r="I15">
         <v>2023</v>
@@ -1148,7 +1160,7 @@
         <v>2015</v>
       </c>
       <c r="O15">
-        <v>72.90000000000001</v>
+        <v>72.69110624794848</v>
       </c>
     </row>
     <row r="16">
@@ -1177,7 +1189,7 @@
         </is>
       </c>
       <c r="H16">
-        <v>0.5</v>
+        <v>0.9583333333333357</v>
       </c>
       <c r="I16">
         <v>2023</v>
@@ -1202,7 +1214,7 @@
         <v>2015</v>
       </c>
       <c r="O16">
-        <v>91.40000000000001</v>
+        <v>91.01666666666667</v>
       </c>
     </row>
     <row r="17">
@@ -1231,7 +1243,7 @@
         </is>
       </c>
       <c r="H17">
-        <v>4.364583333333353</v>
+        <v>5.244904330340312</v>
       </c>
       <c r="I17">
         <v>2023</v>
@@ -1256,7 +1268,7 @@
         <v>2015</v>
       </c>
       <c r="O17">
-        <v>46.6333333333333</v>
+        <v>46.27586206896555</v>
       </c>
     </row>
     <row r="18">
@@ -1285,7 +1297,7 @@
         </is>
       </c>
       <c r="H18">
-        <v>-1.499999999999936</v>
+        <v>-2.289352363752513</v>
       </c>
       <c r="I18">
         <v>2023</v>
@@ -1310,7 +1322,7 @@
         <v>2015</v>
       </c>
       <c r="O18">
-        <v>86.80000000000001</v>
+        <v>86.31571428571428</v>
       </c>
     </row>
     <row r="19">
@@ -1339,7 +1351,7 @@
         </is>
       </c>
       <c r="H19">
-        <v>-4.322916666666522</v>
+        <v>-5.585035079768971</v>
       </c>
       <c r="I19">
         <v>2023</v>
@@ -1364,7 +1376,7 @@
         <v>2015</v>
       </c>
       <c r="O19">
-        <v>85.93333333333335</v>
+        <v>85.4610294117647</v>
       </c>
     </row>
     <row r="20">
@@ -1393,7 +1405,7 @@
         </is>
       </c>
       <c r="H20">
-        <v>2.072916666666579</v>
+        <v>2.553444710110277</v>
       </c>
       <c r="I20">
         <v>2023</v>
@@ -1418,7 +1430,7 @@
         <v>2015</v>
       </c>
       <c r="O20">
-        <v>79.22500000000005</v>
+        <v>78.75665580804073</v>
       </c>
     </row>
     <row r="21">
@@ -1447,7 +1459,7 @@
         </is>
       </c>
       <c r="H21">
-        <v>-0.5833333333333002</v>
+        <v>-0.7594285243741652</v>
       </c>
       <c r="I21">
         <v>2023</v>
@@ -1472,7 +1484,7 @@
         <v>2015</v>
       </c>
       <c r="O21">
-        <v>84.20000000000014</v>
+        <v>83.40592617908406</v>
       </c>
     </row>
     <row r="22">
@@ -1501,7 +1513,7 @@
         </is>
       </c>
       <c r="H22">
-        <v>2.25</v>
+        <v>4.176136363636367</v>
       </c>
       <c r="I22">
         <v>2023</v>
@@ -1526,7 +1538,7 @@
         <v>2015</v>
       </c>
       <c r="O22">
-        <v>89.2</v>
+        <v>88.38818181818182</v>
       </c>
     </row>
     <row r="23">
@@ -1555,7 +1567,7 @@
         </is>
       </c>
       <c r="H23">
-        <v>0.03125</v>
+        <v>0.04032258064516014</v>
       </c>
       <c r="I23">
         <v>2023</v>
@@ -1580,7 +1592,7 @@
         <v>2015</v>
       </c>
       <c r="O23">
-        <v>79.45000000000007</v>
+        <v>79.01794613062134</v>
       </c>
     </row>
     <row r="24">
@@ -1609,7 +1621,7 @@
         </is>
       </c>
       <c r="H24">
-        <v>-1.34375</v>
+        <v>-1.491123808461232</v>
       </c>
       <c r="I24">
         <v>2023</v>
@@ -1634,7 +1646,7 @@
         <v>2015</v>
       </c>
       <c r="O24">
-        <v>78</v>
+        <v>77.34724642056237</v>
       </c>
     </row>
     <row r="25">
@@ -1663,7 +1675,7 @@
         </is>
       </c>
       <c r="H25">
-        <v>-0.9375</v>
+        <v>-0.9836506547032542</v>
       </c>
       <c r="I25">
         <v>2023</v>
@@ -1688,7 +1700,7 @@
         <v>2015</v>
       </c>
       <c r="O25">
-        <v>65.2</v>
+        <v>65.15384615384602</v>
       </c>
     </row>
     <row r="26">
@@ -1717,7 +1729,7 @@
         </is>
       </c>
       <c r="H26">
-        <v>-3.3125</v>
+        <v>-6.281250000000028</v>
       </c>
       <c r="I26">
         <v>2023</v>
@@ -1742,7 +1754,7 @@
         <v>2015</v>
       </c>
       <c r="O26">
-        <v>92.7</v>
+        <v>92.19000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -1770,11 +1782,17 @@
           <t>CHE</t>
         </is>
       </c>
+      <c r="H27">
+        <v>5</v>
+      </c>
       <c r="I27">
         <v>2023</v>
       </c>
       <c r="J27">
-        <v>94.19999999999999</v>
+        <v>94.2</v>
+      </c>
+      <c r="K27">
+        <v>93.80000000000001</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1785,6 +1803,12 @@
         <is>
           <t>Women political empowerment index</t>
         </is>
+      </c>
+      <c r="N27">
+        <v>2015</v>
+      </c>
+      <c r="O27">
+        <v>93.88000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1813,7 +1837,7 @@
         </is>
       </c>
       <c r="H28">
-        <v>4.1875</v>
+        <v>7.70265151515153</v>
       </c>
       <c r="I28">
         <v>2023</v>
@@ -1838,7 +1862,7 @@
         <v>2015</v>
       </c>
       <c r="O28">
-        <v>88.10000000000001</v>
+        <v>87.43000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1867,7 +1891,7 @@
         </is>
       </c>
       <c r="H29">
-        <v>-1.625</v>
+        <v>-1.700906371959</v>
       </c>
       <c r="I29">
         <v>2023</v>
@@ -1892,7 +1916,7 @@
         <v>2015</v>
       </c>
       <c r="O29">
-        <v>66.7</v>
+        <v>66.69230769230762</v>
       </c>
     </row>
     <row r="30">
@@ -1921,7 +1945,7 @@
         </is>
       </c>
       <c r="H30">
-        <v>0.5625</v>
+        <v>0.5904639457270733</v>
       </c>
       <c r="I30">
         <v>2023</v>
@@ -1946,7 +1970,7 @@
         <v>2015</v>
       </c>
       <c r="O30">
-        <v>72.7</v>
+        <v>72.50649086333311</v>
       </c>
     </row>
     <row r="31">
@@ -1975,7 +1999,7 @@
         </is>
       </c>
       <c r="H31">
-        <v>0.2499999999999858</v>
+        <v>0.2831196581196522</v>
       </c>
       <c r="I31">
         <v>2023</v>
@@ -2000,7 +2024,7 @@
         <v>2015</v>
       </c>
       <c r="O31">
-        <v>81.40000000000015</v>
+        <v>81.00713675213679</v>
       </c>
     </row>
     <row r="32">
@@ -2029,7 +2053,7 @@
         </is>
       </c>
       <c r="H32">
-        <v>0.78125</v>
+        <v>0.9403548351158975</v>
       </c>
       <c r="I32">
         <v>2023</v>
@@ -2054,7 +2078,7 @@
         <v>2015</v>
       </c>
       <c r="O32">
-        <v>54.6</v>
+        <v>54.06223484848478</v>
       </c>
     </row>
     <row r="33">
@@ -2083,7 +2107,7 @@
         </is>
       </c>
       <c r="H33">
-        <v>4.375000000000124</v>
+        <v>4.741686314962283</v>
       </c>
       <c r="I33">
         <v>2023</v>
@@ -2108,7 +2132,7 @@
         <v>2015</v>
       </c>
       <c r="O33">
-        <v>34.89999999999993</v>
+        <v>34.63692307692303</v>
       </c>
     </row>
     <row r="34">
@@ -2137,7 +2161,7 @@
         </is>
       </c>
       <c r="H34">
-        <v>0.3749999999999787</v>
+        <v>0.4185744810744794</v>
       </c>
       <c r="I34">
         <v>2023</v>
@@ -2162,7 +2186,7 @@
         <v>2015</v>
       </c>
       <c r="O34">
-        <v>81.00000000000014</v>
+        <v>80.65941391941395</v>
       </c>
     </row>
     <row r="35">
@@ -2191,7 +2215,7 @@
         </is>
       </c>
       <c r="H35">
-        <v>0.875</v>
+        <v>1.073626893939412</v>
       </c>
       <c r="I35">
         <v>2023</v>
@@ -2216,7 +2240,7 @@
         <v>2015</v>
       </c>
       <c r="O35">
-        <v>53.6</v>
+        <v>53.00562499999994</v>
       </c>
     </row>
     <row r="36">
@@ -2245,7 +2269,7 @@
         </is>
       </c>
       <c r="H36">
-        <v>0.9583333333332789</v>
+        <v>1.349611367846478</v>
       </c>
       <c r="I36">
         <v>2023</v>
@@ -2270,7 +2294,7 @@
         <v>2015</v>
       </c>
       <c r="O36">
-        <v>83.20000000000014</v>
+        <v>82.55114812723514</v>
       </c>
     </row>
     <row r="37">
@@ -2299,7 +2323,7 @@
         </is>
       </c>
       <c r="H37">
-        <v>-0.375</v>
+        <v>-1.041666666666664</v>
       </c>
       <c r="I37">
         <v>2023</v>
@@ -2324,7 +2348,7 @@
         <v>2015</v>
       </c>
       <c r="O37">
-        <v>93</v>
+        <v>92.44000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -2353,7 +2377,7 @@
         </is>
       </c>
       <c r="H38">
-        <v>0.71875</v>
+        <v>0.739709851552</v>
       </c>
       <c r="I38">
         <v>2023</v>
@@ -2378,7 +2402,7 @@
         <v>2015</v>
       </c>
       <c r="O38">
-        <v>71</v>
+        <v>70.891282051282</v>
       </c>
     </row>
     <row r="39">
@@ -2407,7 +2431,7 @@
         </is>
       </c>
       <c r="H39">
-        <v>-0.25</v>
+        <v>-0.3229166666666714</v>
       </c>
       <c r="I39">
         <v>2023</v>
@@ -2432,7 +2456,7 @@
         <v>2015</v>
       </c>
       <c r="O39">
-        <v>86.80000000000001</v>
+        <v>86.31571428571428</v>
       </c>
     </row>
     <row r="40">
@@ -2461,7 +2485,7 @@
         </is>
       </c>
       <c r="H40">
-        <v>2.375</v>
+        <v>8.229166666666657</v>
       </c>
       <c r="I40">
         <v>2023</v>
@@ -2486,7 +2510,7 @@
         <v>2015</v>
       </c>
       <c r="O40">
-        <v>92.2</v>
+        <v>91.72</v>
       </c>
     </row>
     <row r="41">
@@ -2557,7 +2581,7 @@
         </is>
       </c>
       <c r="H42">
-        <v>2.250000000000004</v>
+        <v>2.534207026273563</v>
       </c>
       <c r="I42">
         <v>2023</v>
@@ -2582,7 +2606,7 @@
         <v>2015</v>
       </c>
       <c r="O42">
-        <v>56</v>
+        <v>55.52869875222807</v>
       </c>
     </row>
     <row r="43">
@@ -2653,7 +2677,7 @@
         </is>
       </c>
       <c r="H44">
-        <v>1.124999999999936</v>
+        <v>1.585356981881574</v>
       </c>
       <c r="I44">
         <v>2023</v>
@@ -2678,7 +2702,7 @@
         <v>2015</v>
       </c>
       <c r="O44">
-        <v>83.00000000000014</v>
+        <v>82.38370553359687</v>
       </c>
     </row>
     <row r="45">
@@ -2707,7 +2731,7 @@
         </is>
       </c>
       <c r="H45">
-        <v>-4.75</v>
+        <v>-5.213858340635426</v>
       </c>
       <c r="I45">
         <v>2023</v>
@@ -2732,7 +2756,7 @@
         <v>2015</v>
       </c>
       <c r="O45">
-        <v>80.42500000000013</v>
+        <v>80.14483284914326</v>
       </c>
     </row>
     <row r="46">
@@ -2761,7 +2785,7 @@
         </is>
       </c>
       <c r="H46">
-        <v>-2.270833333333258</v>
+        <v>-3.366025690425843</v>
       </c>
       <c r="I46">
         <v>2023</v>
@@ -2786,7 +2810,7 @@
         <v>2015</v>
       </c>
       <c r="O46">
-        <v>87.7</v>
+        <v>87.09076923076927</v>
       </c>
     </row>
     <row r="47">
@@ -2815,7 +2839,7 @@
         </is>
       </c>
       <c r="H47">
-        <v>9.645833333333506</v>
+        <v>10.99685073961445</v>
       </c>
       <c r="I47">
         <v>2023</v>
@@ -2840,7 +2864,7 @@
         <v>2015</v>
       </c>
       <c r="O47">
-        <v>33.09999999999993</v>
+        <v>32.78</v>
       </c>
     </row>
     <row r="48">
@@ -2869,7 +2893,7 @@
         </is>
       </c>
       <c r="H48">
-        <v>1.25</v>
+        <v>1.352339181286517</v>
       </c>
       <c r="I48">
         <v>2023</v>
@@ -2894,7 +2918,7 @@
         <v>2015</v>
       </c>
       <c r="O48">
-        <v>18.6</v>
+        <v>18.46444444444448</v>
       </c>
     </row>
     <row r="49">
@@ -3007,7 +3031,7 @@
         </is>
       </c>
       <c r="H51">
-        <v>1.59375</v>
+        <v>1.695853676116812</v>
       </c>
       <c r="I51">
         <v>2023</v>
@@ -3032,7 +3056,7 @@
         <v>2015</v>
       </c>
       <c r="O51">
-        <v>71.5</v>
+        <v>71.37376518218628</v>
       </c>
     </row>
     <row r="52">
@@ -3103,7 +3127,7 @@
         </is>
       </c>
       <c r="H53">
-        <v>-1.46875</v>
+        <v>-1.496204453441344</v>
       </c>
       <c r="I53">
         <v>2023</v>
@@ -3128,7 +3152,7 @@
         <v>2015</v>
       </c>
       <c r="O53">
-        <v>73.5</v>
+        <v>73.2570981507825</v>
       </c>
     </row>
     <row r="54">
@@ -3156,12 +3180,18 @@
           <t>FRA</t>
         </is>
       </c>
+      <c r="H54">
+        <v>-8.75</v>
+      </c>
       <c r="I54">
         <v>2023</v>
       </c>
       <c r="J54">
         <v>93</v>
       </c>
+      <c r="K54">
+        <v>94</v>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>45.0.0</t>
@@ -3171,6 +3201,12 @@
         <is>
           <t>Women political empowerment index</t>
         </is>
+      </c>
+      <c r="N54">
+        <v>2015</v>
+      </c>
+      <c r="O54">
+        <v>94.08000000000001</v>
       </c>
     </row>
     <row r="55">
@@ -3199,7 +3235,7 @@
         </is>
       </c>
       <c r="H55">
-        <v>1.885416666666607</v>
+        <v>2.28651679668431</v>
       </c>
       <c r="I55">
         <v>2023</v>
@@ -3224,7 +3260,7 @@
         <v>2015</v>
       </c>
       <c r="O55">
-        <v>78.47500000000002</v>
+        <v>77.87777492668626</v>
       </c>
     </row>
     <row r="56">
@@ -3253,7 +3289,7 @@
         </is>
       </c>
       <c r="H56">
-        <v>0.25</v>
+        <v>0.625</v>
       </c>
       <c r="I56">
         <v>2023</v>
@@ -3278,7 +3314,7 @@
         <v>2015</v>
       </c>
       <c r="O56">
-        <v>92.30000000000001</v>
+        <v>91.82000000000001</v>
       </c>
     </row>
     <row r="57">
@@ -3307,7 +3343,7 @@
         </is>
       </c>
       <c r="H57">
-        <v>3.499999999999964</v>
+        <v>6.115003686114356</v>
       </c>
       <c r="I57">
         <v>2023</v>
@@ -3332,7 +3368,7 @@
         <v>2015</v>
       </c>
       <c r="O57">
-        <v>85.20000000000005</v>
+        <v>84.51233574131409</v>
       </c>
     </row>
     <row r="58">
@@ -3361,7 +3397,7 @@
         </is>
       </c>
       <c r="H58">
-        <v>1.791666666666565</v>
+        <v>2.312400953991315</v>
       </c>
       <c r="I58">
         <v>2023</v>
@@ -3386,7 +3422,7 @@
         <v>2015</v>
       </c>
       <c r="O58">
-        <v>81.10000000000015</v>
+        <v>80.74512820512822</v>
       </c>
     </row>
     <row r="59">
@@ -3415,7 +3451,7 @@
         </is>
       </c>
       <c r="H59">
-        <v>0.9375</v>
+        <v>1.185735887096762</v>
       </c>
       <c r="I59">
         <v>2023</v>
@@ -3440,7 +3476,7 @@
         <v>2015</v>
       </c>
       <c r="O59">
-        <v>51.6</v>
+        <v>50.92451612903228</v>
       </c>
     </row>
     <row r="60">
@@ -3469,7 +3505,7 @@
         </is>
       </c>
       <c r="H60">
-        <v>8.156249999999947</v>
+        <v>8.954765375439841</v>
       </c>
       <c r="I60">
         <v>2023</v>
@@ -3494,7 +3530,7 @@
         <v>2015</v>
       </c>
       <c r="O60">
-        <v>58.40000000000001</v>
+        <v>58.05547619047624</v>
       </c>
     </row>
     <row r="61">
@@ -3523,7 +3559,7 @@
         </is>
       </c>
       <c r="H61">
-        <v>-4.03125</v>
+        <v>-4.151817303133122</v>
       </c>
       <c r="I61">
         <v>2023</v>
@@ -3548,7 +3584,7 @@
         <v>2015</v>
       </c>
       <c r="O61">
-        <v>74.90000000000001</v>
+        <v>74.54991848991855</v>
       </c>
     </row>
     <row r="62">
@@ -3577,7 +3613,7 @@
         </is>
       </c>
       <c r="H62">
-        <v>0.9375</v>
+        <v>1.169813049853374</v>
       </c>
       <c r="I62">
         <v>2023</v>
@@ -3602,7 +3638,7 @@
         <v>2015</v>
       </c>
       <c r="O62">
-        <v>52.3</v>
+        <v>51.65169354838709</v>
       </c>
     </row>
     <row r="63">
@@ -3631,7 +3667,7 @@
         </is>
       </c>
       <c r="H63">
-        <v>-2.625</v>
+        <v>-6.645833333333321</v>
       </c>
       <c r="I63">
         <v>2023</v>
@@ -3656,7 +3692,7 @@
         <v>2015</v>
       </c>
       <c r="O63">
-        <v>93.40000000000001</v>
+        <v>92.89333333333333</v>
       </c>
     </row>
     <row r="64">
@@ -3685,7 +3721,7 @@
         </is>
       </c>
       <c r="H64">
-        <v>1.5625</v>
+        <v>1.64945562971878</v>
       </c>
       <c r="I64">
         <v>2023</v>
@@ -3710,7 +3746,7 @@
         <v>2015</v>
       </c>
       <c r="O64">
-        <v>71.10000000000001</v>
+        <v>70.98871794871793</v>
       </c>
     </row>
     <row r="65">
@@ -3739,7 +3775,7 @@
         </is>
       </c>
       <c r="H65">
-        <v>-1.916666666666664</v>
+        <v>-2.927671287046309</v>
       </c>
       <c r="I65">
         <v>2023</v>
@@ -3764,7 +3800,7 @@
         <v>2015</v>
       </c>
       <c r="O65">
-        <v>89.2</v>
+        <v>88.38818181818182</v>
       </c>
     </row>
     <row r="66">
@@ -3793,7 +3829,7 @@
         </is>
       </c>
       <c r="H66">
-        <v>-5.916666666666586</v>
+        <v>-9.853654909033331</v>
       </c>
       <c r="I66">
         <v>2023</v>
@@ -3818,7 +3854,7 @@
         <v>2015</v>
       </c>
       <c r="O66">
-        <v>91.40000000000001</v>
+        <v>91.01666666666667</v>
       </c>
     </row>
     <row r="67">
@@ -3847,7 +3883,7 @@
         </is>
       </c>
       <c r="H67">
-        <v>2.333333333333286</v>
+        <v>2.797328166686867</v>
       </c>
       <c r="I67">
         <v>2023</v>
@@ -3872,7 +3908,7 @@
         <v>2015</v>
       </c>
       <c r="O67">
-        <v>76.5</v>
+        <v>76.00541380188436</v>
       </c>
     </row>
     <row r="68">
@@ -3901,7 +3937,7 @@
         </is>
       </c>
       <c r="H68">
-        <v>3.875</v>
+        <v>8.104166666666686</v>
       </c>
       <c r="I68">
         <v>2023</v>
@@ -3926,7 +3962,7 @@
         <v>2015</v>
       </c>
       <c r="O68">
-        <v>90.2</v>
+        <v>89.95999999999999</v>
       </c>
     </row>
     <row r="69">
@@ -3955,7 +3991,7 @@
         </is>
       </c>
       <c r="H69">
-        <v>-5.125000000000146</v>
+        <v>-5.592150505943728</v>
       </c>
       <c r="I69">
         <v>2023</v>
@@ -3980,7 +4016,7 @@
         <v>2015</v>
       </c>
       <c r="O69">
-        <v>45.83333333333321</v>
+        <v>45.65517241379311</v>
       </c>
     </row>
     <row r="70">
@@ -4034,7 +4070,7 @@
         <v>2015</v>
       </c>
       <c r="O70">
-        <v>87.10000000000001</v>
+        <v>86.56989010989011</v>
       </c>
     </row>
     <row r="71">
@@ -4063,7 +4099,7 @@
         </is>
       </c>
       <c r="H71">
-        <v>-1.46875</v>
+        <v>-1.589626569889674</v>
       </c>
       <c r="I71">
         <v>2023</v>
@@ -4088,7 +4124,7 @@
         <v>2015</v>
       </c>
       <c r="O71">
-        <v>77.2</v>
+        <v>76.63461962057546</v>
       </c>
     </row>
     <row r="72">
@@ -4142,7 +4178,7 @@
         <v>2015</v>
       </c>
       <c r="O72">
-        <v>70.3</v>
+        <v>70.21653846153831</v>
       </c>
     </row>
     <row r="73">
@@ -4171,7 +4207,7 @@
         </is>
       </c>
       <c r="H73">
-        <v>2.5</v>
+        <v>6.979166666666657</v>
       </c>
       <c r="I73">
         <v>2023</v>
@@ -4196,7 +4232,7 @@
         <v>2015</v>
       </c>
       <c r="O73">
-        <v>91.7</v>
+        <v>91.30000000000001</v>
       </c>
     </row>
     <row r="74">
@@ -4225,7 +4261,7 @@
         </is>
       </c>
       <c r="H74">
-        <v>-1.083333333333364</v>
+        <v>-1.205484330484364</v>
       </c>
       <c r="I74">
         <v>2023</v>
@@ -4250,7 +4286,7 @@
         <v>2015</v>
       </c>
       <c r="O74">
-        <v>37.99999999999993</v>
+        <v>37.79185185185178</v>
       </c>
     </row>
     <row r="75">
@@ -4279,7 +4315,7 @@
         </is>
       </c>
       <c r="H75">
-        <v>0.375</v>
+        <v>0.4569128787878896</v>
       </c>
       <c r="I75">
         <v>2023</v>
@@ -4304,7 +4340,7 @@
         <v>2015</v>
       </c>
       <c r="O75">
-        <v>54.5</v>
+        <v>53.95598484848477</v>
       </c>
     </row>
     <row r="76">
@@ -4333,7 +4369,7 @@
         </is>
       </c>
       <c r="H76">
-        <v>-4.3125</v>
+        <v>-9.180555555555571</v>
       </c>
       <c r="I76">
         <v>2023</v>
@@ -4358,7 +4394,7 @@
         <v>2015</v>
       </c>
       <c r="O76">
-        <v>93.30000000000001</v>
+        <v>92.74000000000001</v>
       </c>
     </row>
     <row r="77">
@@ -4387,7 +4423,7 @@
         </is>
       </c>
       <c r="H77">
-        <v>-0.3125</v>
+        <v>-0.6388888888888857</v>
       </c>
       <c r="I77">
         <v>2023</v>
@@ -4412,7 +4448,7 @@
         <v>2015</v>
       </c>
       <c r="O77">
-        <v>89.65000000000001</v>
+        <v>88.99555555555557</v>
       </c>
     </row>
     <row r="78">
@@ -4441,7 +4477,7 @@
         </is>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>4.583333333333336</v>
       </c>
       <c r="I78">
         <v>2023</v>
@@ -4466,7 +4502,7 @@
         <v>2015</v>
       </c>
       <c r="O78">
-        <v>93.40000000000001</v>
+        <v>92.82666666666668</v>
       </c>
     </row>
     <row r="79">
@@ -4537,7 +4573,7 @@
         </is>
       </c>
       <c r="H80">
-        <v>-0.6875</v>
+        <v>-0.7051282051282612</v>
       </c>
       <c r="I80">
         <v>2023</v>
@@ -4591,7 +4627,7 @@
         </is>
       </c>
       <c r="H81">
-        <v>0.5729166666666359</v>
+        <v>0.6352758831207055</v>
       </c>
       <c r="I81">
         <v>2023</v>
@@ -4616,7 +4652,7 @@
         <v>2015</v>
       </c>
       <c r="O81">
-        <v>80.42500000000013</v>
+        <v>80.14483284914326</v>
       </c>
     </row>
     <row r="82">
@@ -4645,7 +4681,7 @@
         </is>
       </c>
       <c r="H82">
-        <v>-0.9687499999999645</v>
+        <v>-1.15384352237799</v>
       </c>
       <c r="I82">
         <v>2023</v>
@@ -4670,7 +4706,7 @@
         <v>2015</v>
       </c>
       <c r="O82">
-        <v>82.00000000000014</v>
+        <v>81.52250836120407</v>
       </c>
     </row>
     <row r="83">
@@ -4699,7 +4735,7 @@
         </is>
       </c>
       <c r="H83">
-        <v>0.71875</v>
+        <v>0.861724519353217</v>
       </c>
       <c r="I83">
         <v>2023</v>
@@ -4724,7 +4760,7 @@
         <v>2015</v>
       </c>
       <c r="O83">
-        <v>77.10000000000001</v>
+        <v>76.54604819200404</v>
       </c>
     </row>
     <row r="84">
@@ -4753,7 +4789,7 @@
         </is>
       </c>
       <c r="H84">
-        <v>-2.104166666666622</v>
+        <v>-2.533042452401162</v>
       </c>
       <c r="I84">
         <v>2023</v>
@@ -4778,7 +4814,7 @@
         <v>2015</v>
       </c>
       <c r="O84">
-        <v>82.40000000000015</v>
+        <v>81.86773913043484</v>
       </c>
     </row>
     <row r="85">
@@ -4807,7 +4843,7 @@
         </is>
       </c>
       <c r="H85">
-        <v>-2.187500000000004</v>
+        <v>-2.517018785401149</v>
       </c>
       <c r="I85">
         <v>2023</v>
@@ -4832,7 +4868,7 @@
         <v>2015</v>
       </c>
       <c r="O85">
-        <v>61.90000000000001</v>
+        <v>61.73479374110966</v>
       </c>
     </row>
     <row r="86">
@@ -4861,7 +4897,7 @@
         </is>
       </c>
       <c r="H86">
-        <v>0.75</v>
+        <v>1.254370629370626</v>
       </c>
       <c r="I86">
         <v>2023</v>
@@ -4886,7 +4922,7 @@
         <v>2015</v>
       </c>
       <c r="O86">
-        <v>87.80000000000001</v>
+        <v>87.17615384615387</v>
       </c>
     </row>
     <row r="87">
@@ -4915,7 +4951,7 @@
         </is>
       </c>
       <c r="H87">
-        <v>-0.4166666666666785</v>
+        <v>-0.4464285714285765</v>
       </c>
       <c r="I87">
         <v>2023</v>
@@ -4940,7 +4976,7 @@
         <v>2015</v>
       </c>
       <c r="O87">
-        <v>43.49999999999993</v>
+        <v>43.41999999999989</v>
       </c>
     </row>
     <row r="88">
@@ -4969,7 +5005,7 @@
         </is>
       </c>
       <c r="H88">
-        <v>0.875</v>
+        <v>1.134492607526845</v>
       </c>
       <c r="I88">
         <v>2023</v>
@@ -4994,7 +5030,7 @@
         <v>2015</v>
       </c>
       <c r="O88">
-        <v>50</v>
+        <v>49.26333333333343</v>
       </c>
     </row>
     <row r="89">
@@ -5023,7 +5059,7 @@
         </is>
       </c>
       <c r="H89">
-        <v>1.750000000000004</v>
+        <v>1.903479137031681</v>
       </c>
       <c r="I89">
         <v>2023</v>
@@ -5048,7 +5084,7 @@
         <v>2015</v>
       </c>
       <c r="O89">
-        <v>58.8</v>
+        <v>58.47833333333339</v>
       </c>
     </row>
     <row r="90">
@@ -5077,7 +5113,7 @@
         </is>
       </c>
       <c r="H90">
-        <v>-0.6249999999999645</v>
+        <v>-1.010728414172682</v>
       </c>
       <c r="I90">
         <v>2023</v>
@@ -5102,7 +5138,7 @@
         <v>2015</v>
       </c>
       <c r="O90">
-        <v>85.8666666666667</v>
+        <v>85.37279411764706</v>
       </c>
     </row>
     <row r="91">
@@ -5131,7 +5167,7 @@
         </is>
       </c>
       <c r="H91">
-        <v>1.385416666666696</v>
+        <v>1.525862068965523</v>
       </c>
       <c r="I91">
         <v>2023</v>
@@ -5156,7 +5192,7 @@
         <v>2015</v>
       </c>
       <c r="O91">
-        <v>45.19999999999993</v>
+        <v>45.13793103448266</v>
       </c>
     </row>
     <row r="92">
@@ -5185,7 +5221,7 @@
         </is>
       </c>
       <c r="H92">
-        <v>-1.875</v>
+        <v>-1.940061139074309</v>
       </c>
       <c r="I92">
         <v>2023</v>
@@ -5210,7 +5246,7 @@
         <v>2015</v>
       </c>
       <c r="O92">
-        <v>75.3</v>
+        <v>74.91748605748607</v>
       </c>
     </row>
     <row r="93">
@@ -5239,7 +5275,7 @@
         </is>
       </c>
       <c r="H93">
-        <v>0.4999999999999716</v>
+        <v>0.6800536420101437</v>
       </c>
       <c r="I93">
         <v>2023</v>
@@ -5264,7 +5300,7 @@
         <v>2015</v>
       </c>
       <c r="O93">
-        <v>83.40000000000015</v>
+        <v>82.72143798230759</v>
       </c>
     </row>
     <row r="94">
@@ -5293,7 +5329,7 @@
         </is>
       </c>
       <c r="H94">
-        <v>3.25</v>
+        <v>9.562499999999993</v>
       </c>
       <c r="I94">
         <v>2023</v>
@@ -5318,7 +5354,7 @@
         <v>2015</v>
       </c>
       <c r="O94">
-        <v>91.40000000000001</v>
+        <v>91.01666666666667</v>
       </c>
     </row>
     <row r="95">
@@ -5347,7 +5383,7 @@
         </is>
       </c>
       <c r="H95">
-        <v>2.625</v>
+        <v>4.743055555555571</v>
       </c>
       <c r="I95">
         <v>2023</v>
@@ -5372,7 +5408,7 @@
         <v>2015</v>
       </c>
       <c r="O95">
-        <v>89.7</v>
+        <v>89.08444444444446</v>
       </c>
     </row>
     <row r="96">
@@ -5443,7 +5479,7 @@
         </is>
       </c>
       <c r="H97">
-        <v>1.53125</v>
+        <v>1.721152422777784</v>
       </c>
       <c r="I97">
         <v>2023</v>
@@ -5468,7 +5504,7 @@
         <v>2015</v>
       </c>
       <c r="O97">
-        <v>73.8</v>
+        <v>73.53460565829002</v>
       </c>
     </row>
     <row r="98">
@@ -5497,7 +5533,7 @@
         </is>
       </c>
       <c r="H98">
-        <v>4.25</v>
+        <v>7.952651515151537</v>
       </c>
       <c r="I98">
         <v>2023</v>
@@ -5522,7 +5558,7 @@
         <v>2015</v>
       </c>
       <c r="O98">
-        <v>88.40000000000001</v>
+        <v>87.70454545454545</v>
       </c>
     </row>
     <row r="99">
@@ -5551,7 +5587,7 @@
         </is>
       </c>
       <c r="H99">
-        <v>-2.583333333333293</v>
+        <v>-3.062117956476655</v>
       </c>
       <c r="I99">
         <v>2023</v>
@@ -5576,7 +5612,7 @@
         <v>2015</v>
       </c>
       <c r="O99">
-        <v>82.20000000000014</v>
+        <v>81.69173913043481</v>
       </c>
     </row>
     <row r="100">
@@ -5605,7 +5641,7 @@
         </is>
       </c>
       <c r="H100">
-        <v>2.843750000000004</v>
+        <v>3.267174031855717</v>
       </c>
       <c r="I100">
         <v>2023</v>
@@ -5630,7 +5666,7 @@
         <v>2015</v>
       </c>
       <c r="O100">
-        <v>54</v>
+        <v>53.42473484848477</v>
       </c>
     </row>
     <row r="101">
@@ -5659,7 +5695,7 @@
         </is>
       </c>
       <c r="H101">
-        <v>0.8333333333333286</v>
+        <v>1.069896611314149</v>
       </c>
       <c r="I101">
         <v>2023</v>
@@ -5684,7 +5720,7 @@
         <v>2015</v>
       </c>
       <c r="O101">
-        <v>78.7</v>
+        <v>78.14141129032259</v>
       </c>
     </row>
     <row r="102">
@@ -5713,7 +5749,7 @@
         </is>
       </c>
       <c r="H102">
-        <v>-0.8958333333333073</v>
+        <v>-1.364174836601293</v>
       </c>
       <c r="I102">
         <v>2023</v>
@@ -5738,7 +5774,7 @@
         <v>2015</v>
       </c>
       <c r="O102">
-        <v>86.90000000000001</v>
+        <v>86.40238095238095</v>
       </c>
     </row>
     <row r="103">
@@ -5767,7 +5803,7 @@
         </is>
       </c>
       <c r="H103">
-        <v>0.375</v>
+        <v>0.3956258890469115</v>
       </c>
       <c r="I103">
         <v>2023</v>
@@ -5792,7 +5828,7 @@
         <v>2015</v>
       </c>
       <c r="O103">
-        <v>73.3</v>
+        <v>73.06762446657198</v>
       </c>
     </row>
     <row r="104">
@@ -5821,7 +5857,7 @@
         </is>
       </c>
       <c r="H104">
-        <v>5.708333333333321</v>
+        <v>9.985854219310127</v>
       </c>
       <c r="I104">
         <v>2023</v>
@@ -5846,7 +5882,7 @@
         <v>2015</v>
       </c>
       <c r="O104">
-        <v>85.8666666666667</v>
+        <v>85.37279411764706</v>
       </c>
     </row>
     <row r="105">
@@ -5875,7 +5911,7 @@
         </is>
       </c>
       <c r="H105">
-        <v>-8.635416666666803</v>
+        <v>-9.829553634817312</v>
       </c>
       <c r="I105">
         <v>2023</v>
@@ -5900,7 +5936,7 @@
         <v>2015</v>
       </c>
       <c r="O105">
-        <v>61.2</v>
+        <v>61.00216216216231</v>
       </c>
     </row>
     <row r="106">
@@ -5929,7 +5965,7 @@
         </is>
       </c>
       <c r="H106">
-        <v>0.5833333333333002</v>
+        <v>0.8795426065163028</v>
       </c>
       <c r="I106">
         <v>2023</v>
@@ -5954,7 +5990,7 @@
         <v>2015</v>
       </c>
       <c r="O106">
-        <v>84.40000000000015</v>
+        <v>83.57345864661653</v>
       </c>
     </row>
     <row r="107">
@@ -5983,7 +6019,7 @@
         </is>
       </c>
       <c r="H107">
-        <v>-4.312499999999851</v>
+        <v>-6.133886754482518</v>
       </c>
       <c r="I107">
         <v>2023</v>
@@ -6008,7 +6044,7 @@
         <v>2015</v>
       </c>
       <c r="O107">
-        <v>88.90000000000001</v>
+        <v>88.13636363636363</v>
       </c>
     </row>
     <row r="108">
@@ -6037,7 +6073,7 @@
         </is>
       </c>
       <c r="H108">
-        <v>-0.125</v>
+        <v>-0.1439075630252091</v>
       </c>
       <c r="I108">
         <v>2023</v>
@@ -6062,7 +6098,7 @@
         <v>2015</v>
       </c>
       <c r="O108">
-        <v>77.5</v>
+        <v>76.90293894830657</v>
       </c>
     </row>
     <row r="109">
@@ -6116,7 +6152,7 @@
         <v>2015</v>
       </c>
       <c r="O109">
-        <v>67.5</v>
+        <v>67.49750000000003</v>
       </c>
     </row>
     <row r="110">
@@ -6145,7 +6181,7 @@
         </is>
       </c>
       <c r="H110">
-        <v>-2.020833333333222</v>
+        <v>-2.536636110848967</v>
       </c>
       <c r="I110">
         <v>2023</v>
@@ -6170,7 +6206,7 @@
         <v>2015</v>
       </c>
       <c r="O110">
-        <v>85.00000000000009</v>
+        <v>84.25540935672517</v>
       </c>
     </row>
     <row r="111">
@@ -6199,7 +6235,7 @@
         </is>
       </c>
       <c r="H111">
-        <v>0.1875</v>
+        <v>0.2543103448275872</v>
       </c>
       <c r="I111">
         <v>2023</v>
@@ -6224,7 +6260,7 @@
         <v>2015</v>
       </c>
       <c r="O111">
-        <v>79.90000000000015</v>
+        <v>79.54000547345375</v>
       </c>
     </row>
     <row r="112">
@@ -6253,7 +6289,7 @@
         </is>
       </c>
       <c r="H112">
-        <v>4.239583333333314</v>
+        <v>4.732859294981175</v>
       </c>
       <c r="I112">
         <v>2023</v>
@@ -6278,7 +6314,7 @@
         <v>2015</v>
       </c>
       <c r="O112">
-        <v>68.8</v>
+        <v>68.7649999999999</v>
       </c>
     </row>
     <row r="113">
@@ -6307,7 +6343,7 @@
         </is>
       </c>
       <c r="H113">
-        <v>-0.1666666666666572</v>
+        <v>-0.2777777777777715</v>
       </c>
       <c r="I113">
         <v>2023</v>
@@ -6332,7 +6368,7 @@
         <v>2015</v>
       </c>
       <c r="O113">
-        <v>85.6666666666667</v>
+        <v>85.11299019607844</v>
       </c>
     </row>
     <row r="114">
@@ -6361,7 +6397,7 @@
         </is>
       </c>
       <c r="H114">
-        <v>-1.84375</v>
+        <v>-2.000421657155371</v>
       </c>
       <c r="I114">
         <v>2023</v>
@@ -6386,7 +6422,7 @@
         <v>2015</v>
       </c>
       <c r="O114">
-        <v>77.80000000000001</v>
+        <v>77.17077583232705</v>
       </c>
     </row>
     <row r="115">
@@ -6415,7 +6451,7 @@
         </is>
       </c>
       <c r="H115">
-        <v>-0.53125</v>
+        <v>-0.5762999841946979</v>
       </c>
       <c r="I115">
         <v>2023</v>
@@ -6440,7 +6476,7 @@
         <v>2015</v>
       </c>
       <c r="O115">
-        <v>75.90000000000001</v>
+        <v>75.46495798319326</v>
       </c>
     </row>
     <row r="116">
@@ -6469,7 +6505,7 @@
         </is>
       </c>
       <c r="H116">
-        <v>-5.5625</v>
+        <v>-5.931243906771059</v>
       </c>
       <c r="I116">
         <v>2023</v>
@@ -6494,7 +6530,7 @@
         <v>2015</v>
       </c>
       <c r="O116">
-        <v>79.30000000000008</v>
+        <v>78.84375258223426</v>
       </c>
     </row>
     <row r="117">
@@ -6523,7 +6559,7 @@
         </is>
       </c>
       <c r="H117">
-        <v>-1.125</v>
+        <v>-2.166666666666671</v>
       </c>
       <c r="I117">
         <v>2023</v>
@@ -6548,7 +6584,7 @@
         <v>2015</v>
       </c>
       <c r="O117">
-        <v>92.2</v>
+        <v>91.72</v>
       </c>
     </row>
     <row r="118">
@@ -6619,7 +6655,7 @@
         </is>
       </c>
       <c r="H119">
-        <v>-0.4270833333333286</v>
+        <v>-0.5532635467980285</v>
       </c>
       <c r="I119">
         <v>2023</v>
@@ -6644,7 +6680,7 @@
         <v>2015</v>
       </c>
       <c r="O119">
-        <v>80.70000000000014</v>
+        <v>80.40227106227114</v>
       </c>
     </row>
     <row r="120">
@@ -6715,7 +6751,7 @@
         </is>
       </c>
       <c r="H121">
-        <v>-0.1666666666666714</v>
+        <v>-0.1785714285714306</v>
       </c>
       <c r="I121">
         <v>2023</v>
@@ -6740,7 +6776,7 @@
         <v>2015</v>
       </c>
       <c r="O121">
-        <v>39.89999999999993</v>
+        <v>39.73999999999999</v>
       </c>
     </row>
     <row r="122">
@@ -6769,7 +6805,7 @@
         </is>
       </c>
       <c r="H122">
-        <v>-1.281250000000004</v>
+        <v>-1.388493756914748</v>
       </c>
       <c r="I122">
         <v>2023</v>
@@ -6794,7 +6830,7 @@
         <v>2015</v>
       </c>
       <c r="O122">
-        <v>63.7</v>
+        <v>63.60157894736831</v>
       </c>
     </row>
     <row r="123">
@@ -6823,7 +6859,7 @@
         </is>
       </c>
       <c r="H123">
-        <v>-1.37499999999995</v>
+        <v>-1.651610271757619</v>
       </c>
       <c r="I123">
         <v>2023</v>
@@ -6848,7 +6884,7 @@
         <v>2015</v>
       </c>
       <c r="O123">
-        <v>82.60000000000015</v>
+        <v>82.03720553359686</v>
       </c>
     </row>
     <row r="124">
@@ -6877,7 +6913,7 @@
         </is>
       </c>
       <c r="H124">
-        <v>1.395833333333258</v>
+        <v>1.650578328052063</v>
       </c>
       <c r="I124">
         <v>2023</v>
@@ -6902,7 +6938,7 @@
         <v>2015</v>
       </c>
       <c r="O124">
-        <v>80.35000000000011</v>
+        <v>80.05862595259154</v>
       </c>
     </row>
     <row r="125">
@@ -6931,7 +6967,7 @@
         </is>
       </c>
       <c r="H125">
-        <v>-1.729166666666572</v>
+        <v>-2.600390736611516</v>
       </c>
       <c r="I125">
         <v>2023</v>
@@ -6956,7 +6992,7 @@
         <v>2015</v>
       </c>
       <c r="O125">
-        <v>86.30000000000001</v>
+        <v>85.89083333333332</v>
       </c>
     </row>
     <row r="126">
@@ -6985,7 +7021,7 @@
         </is>
       </c>
       <c r="H126">
-        <v>0.46875</v>
+        <v>0.6048387096774022</v>
       </c>
       <c r="I126">
         <v>2023</v>
@@ -7010,7 +7046,7 @@
         <v>2015</v>
       </c>
       <c r="O126">
-        <v>50.5</v>
+        <v>49.78903225806455</v>
       </c>
     </row>
     <row r="127">
@@ -7039,7 +7075,7 @@
         </is>
       </c>
       <c r="H127">
-        <v>-7.5</v>
+        <v>-17.359015984016</v>
       </c>
       <c r="I127">
         <v>2023</v>
@@ -7064,7 +7100,7 @@
         <v>2015</v>
       </c>
       <c r="O127">
-        <v>93.40000000000001</v>
+        <v>93.46000000000001</v>
       </c>
     </row>
     <row r="128">
@@ -7093,7 +7129,7 @@
         </is>
       </c>
       <c r="H128">
-        <v>0.9375000000000178</v>
+        <v>1.002083333333346</v>
       </c>
       <c r="I128">
         <v>2023</v>
@@ -7118,7 +7154,7 @@
         <v>2015</v>
       </c>
       <c r="O128">
-        <v>30.04999999999997</v>
+        <v>29.89583333333328</v>
       </c>
     </row>
     <row r="129">
@@ -7147,7 +7183,7 @@
         </is>
       </c>
       <c r="H129">
-        <v>-4.75</v>
+        <v>-11.54166666666669</v>
       </c>
       <c r="I129">
         <v>2023</v>
@@ -7172,7 +7208,7 @@
         <v>2015</v>
       </c>
       <c r="O129">
-        <v>93.40000000000001</v>
+        <v>93.26000000000001</v>
       </c>
     </row>
     <row r="130">
@@ -7201,7 +7237,7 @@
         </is>
       </c>
       <c r="H130">
-        <v>0.34375</v>
+        <v>0.3645092460881685</v>
       </c>
       <c r="I130">
         <v>2023</v>
@@ -7226,7 +7262,7 @@
         <v>2015</v>
       </c>
       <c r="O130">
-        <v>73.60000000000001</v>
+        <v>73.3503951319742</v>
       </c>
     </row>
     <row r="131">
@@ -7255,7 +7291,7 @@
         </is>
       </c>
       <c r="H131">
-        <v>-1.302083333333343</v>
+        <v>-1.611651835372562</v>
       </c>
       <c r="I131">
         <v>2023</v>
@@ -7280,7 +7316,7 @@
         <v>2015</v>
       </c>
       <c r="O131">
-        <v>51.6</v>
+        <v>50.92451612903228</v>
       </c>
     </row>
     <row r="132">
@@ -7309,7 +7345,7 @@
         </is>
       </c>
       <c r="H132">
-        <v>-1.416666666666696</v>
+        <v>-1.542628205128221</v>
       </c>
       <c r="I132">
         <v>2023</v>
@@ -7334,7 +7370,7 @@
         <v>2015</v>
       </c>
       <c r="O132">
-        <v>33.29999999999993</v>
+        <v>32.98</v>
       </c>
     </row>
     <row r="133">
@@ -7363,7 +7399,7 @@
         </is>
       </c>
       <c r="H133">
-        <v>1.375</v>
+        <v>2.046989468864474</v>
       </c>
       <c r="I133">
         <v>2023</v>
@@ -7388,7 +7424,7 @@
         <v>2015</v>
       </c>
       <c r="O133">
-        <v>86.5</v>
+        <v>86.06113095238094</v>
       </c>
     </row>
     <row r="134">
@@ -7417,7 +7453,7 @@
         </is>
       </c>
       <c r="H134">
-        <v>-3.906250000000004</v>
+        <v>-4.060530419083072</v>
       </c>
       <c r="I134">
         <v>2023</v>
@@ -7442,7 +7478,7 @@
         <v>2015</v>
       </c>
       <c r="O134">
-        <v>72</v>
+        <v>71.84812415654528</v>
       </c>
     </row>
     <row r="135">
@@ -7471,7 +7507,7 @@
         </is>
       </c>
       <c r="H135">
-        <v>-7.166666666666544</v>
+        <v>-8.25740787230437</v>
       </c>
       <c r="I135">
         <v>2023</v>
@@ -7496,7 +7532,7 @@
         <v>2015</v>
       </c>
       <c r="O135">
-        <v>85.3333333333334</v>
+        <v>84.68075679394569</v>
       </c>
     </row>
     <row r="136">
@@ -7525,7 +7561,7 @@
         </is>
       </c>
       <c r="H136">
-        <v>4.562500000000053</v>
+        <v>4.472010869565224</v>
       </c>
       <c r="I136">
         <v>2023</v>
@@ -7550,7 +7586,7 @@
         <v>2015</v>
       </c>
       <c r="O136">
-        <v>25.7</v>
+        <v>25.94173913043477</v>
       </c>
     </row>
     <row r="137">
@@ -7579,7 +7615,7 @@
         </is>
       </c>
       <c r="H137">
-        <v>-5.604166666666806</v>
+        <v>-6.093210724460807</v>
       </c>
       <c r="I137">
         <v>2023</v>
@@ -7604,7 +7640,7 @@
         <v>2015</v>
       </c>
       <c r="O137">
-        <v>42.59999999999993</v>
+        <v>42.48785714285707</v>
       </c>
     </row>
     <row r="138">
@@ -7633,7 +7669,7 @@
         </is>
       </c>
       <c r="H138">
-        <v>1.458333333333307</v>
+        <v>2.169577767004235</v>
       </c>
       <c r="I138">
         <v>2023</v>
@@ -7658,7 +7694,7 @@
         <v>2015</v>
       </c>
       <c r="O138">
-        <v>85.4666666666667</v>
+        <v>84.85385620915036</v>
       </c>
     </row>
     <row r="139">
@@ -7687,7 +7723,7 @@
         </is>
       </c>
       <c r="H139">
-        <v>-0.9999999999999432</v>
+        <v>-1.15506715506713</v>
       </c>
       <c r="I139">
         <v>2023</v>
@@ -7712,7 +7748,7 @@
         <v>2015</v>
       </c>
       <c r="O139">
-        <v>83.10000000000015</v>
+        <v>82.46781479390179</v>
       </c>
     </row>
     <row r="140">
@@ -7741,7 +7777,7 @@
         </is>
       </c>
       <c r="H140">
-        <v>6.73958333333335</v>
+        <v>7.720462011433369</v>
       </c>
       <c r="I140">
         <v>2023</v>
@@ -7766,7 +7802,7 @@
         <v>2015</v>
       </c>
       <c r="O140">
-        <v>47.0333333333333</v>
+        <v>46.58620689655181</v>
       </c>
     </row>
     <row r="141">
@@ -7795,7 +7831,7 @@
         </is>
       </c>
       <c r="H141">
-        <v>1.291666666666593</v>
+        <v>1.543148276843894</v>
       </c>
       <c r="I141">
         <v>2023</v>
@@ -7820,7 +7856,7 @@
         <v>2015</v>
       </c>
       <c r="O141">
-        <v>80.80000000000015</v>
+        <v>80.48798534798541</v>
       </c>
     </row>
     <row r="142">
@@ -7849,7 +7885,7 @@
         </is>
       </c>
       <c r="H142">
-        <v>-7.468750000000004</v>
+        <v>-8.147870247804384</v>
       </c>
       <c r="I142">
         <v>2023</v>
@@ -7874,7 +7910,7 @@
         <v>2015</v>
       </c>
       <c r="O142">
-        <v>80.12500000000013</v>
+        <v>79.80000526293634</v>
       </c>
     </row>
     <row r="143">
@@ -7903,7 +7939,7 @@
         </is>
       </c>
       <c r="H143">
-        <v>5.854166666666799</v>
+        <v>6.242020248270318</v>
       </c>
       <c r="I143">
         <v>2023</v>
@@ -7928,7 +7964,7 @@
         <v>2015</v>
       </c>
       <c r="O143">
-        <v>28.1</v>
+        <v>28.43750000000001</v>
       </c>
     </row>
     <row r="144">
@@ -7957,7 +7993,7 @@
         </is>
       </c>
       <c r="H144">
-        <v>2.4375</v>
+        <v>4.126377095127104</v>
       </c>
       <c r="I144">
         <v>2023</v>
@@ -7982,7 +8018,7 @@
         <v>2015</v>
       </c>
       <c r="O144">
-        <v>86.40000000000001</v>
+        <v>85.97833333333332</v>
       </c>
     </row>
     <row r="145">
@@ -8011,7 +8047,7 @@
         </is>
       </c>
       <c r="H145">
-        <v>-1.250000000000036</v>
+        <v>-1.331588669950747</v>
       </c>
       <c r="I145">
         <v>2023</v>
@@ -8036,7 +8072,7 @@
         <v>2015</v>
       </c>
       <c r="O145">
-        <v>43.99999999999993</v>
+        <v>43.91999999999987</v>
       </c>
     </row>
     <row r="146">
@@ -8065,7 +8101,7 @@
         </is>
       </c>
       <c r="H146">
-        <v>2.020833333333265</v>
+        <v>3.010131584531742</v>
       </c>
       <c r="I146">
         <v>2023</v>
@@ -8090,7 +8126,7 @@
         <v>2015</v>
       </c>
       <c r="O146">
-        <v>84.10000000000015</v>
+        <v>83.31989177489177</v>
       </c>
     </row>
     <row r="147">
@@ -8119,7 +8155,7 @@
         </is>
       </c>
       <c r="H147">
-        <v>1.874999999999972</v>
+        <v>2.839983749910211</v>
       </c>
       <c r="I147">
         <v>2023</v>
@@ -8144,7 +8180,7 @@
         <v>2015</v>
       </c>
       <c r="O147">
-        <v>85.40000000000005</v>
+        <v>84.76496732026146</v>
       </c>
     </row>
     <row r="148">
@@ -8173,7 +8209,7 @@
         </is>
       </c>
       <c r="H148">
-        <v>1.4375</v>
+        <v>2.788690476190467</v>
       </c>
       <c r="I148">
         <v>2023</v>
@@ -8198,7 +8234,7 @@
         <v>2015</v>
       </c>
       <c r="O148">
-        <v>89.55000000000001</v>
+        <v>88.82666666666668</v>
       </c>
     </row>
     <row r="149">
@@ -8226,11 +8262,17 @@
           <t>SVN</t>
         </is>
       </c>
+      <c r="H149">
+        <v>-6.25</v>
+      </c>
       <c r="I149">
         <v>2023</v>
       </c>
       <c r="J149">
-        <v>93.8</v>
+        <v>93.80000000000001</v>
+      </c>
+      <c r="K149">
+        <v>94.30000000000001</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -8241,6 +8283,9 @@
         <is>
           <t>Women political empowerment index</t>
         </is>
+      </c>
+      <c r="N149">
+        <v>2015</v>
       </c>
     </row>
     <row r="150">
@@ -8311,7 +8356,7 @@
         </is>
       </c>
       <c r="H151">
-        <v>-1.500000000000043</v>
+        <v>-1.714743589743609</v>
       </c>
       <c r="I151">
         <v>2023</v>
@@ -8336,7 +8381,7 @@
         <v>2015</v>
       </c>
       <c r="O151">
-        <v>36.39999999999993</v>
+        <v>36.15999999999995</v>
       </c>
     </row>
     <row r="152">
@@ -8365,7 +8410,7 @@
         </is>
       </c>
       <c r="H152">
-        <v>2.5</v>
+        <v>4.630681818181834</v>
       </c>
       <c r="I152">
         <v>2023</v>
@@ -8390,7 +8435,7 @@
         <v>2015</v>
       </c>
       <c r="O152">
-        <v>88.80000000000001</v>
+        <v>88.04545454545453</v>
       </c>
     </row>
     <row r="153">
@@ -8419,7 +8464,7 @@
         </is>
       </c>
       <c r="H153">
-        <v>-0.833333333333357</v>
+        <v>-0.961538461538467</v>
       </c>
       <c r="I153">
         <v>2023</v>
@@ -8444,7 +8489,7 @@
         <v>2015</v>
       </c>
       <c r="O153">
-        <v>35.19999999999993</v>
+        <v>34.9484615384615</v>
       </c>
     </row>
     <row r="154">
@@ -8473,7 +8518,7 @@
         </is>
       </c>
       <c r="H154">
-        <v>1.687500000000004</v>
+        <v>1.871855961445689</v>
       </c>
       <c r="I154">
         <v>2023</v>
@@ -8498,7 +8543,7 @@
         <v>2015</v>
       </c>
       <c r="O154">
-        <v>57.7</v>
+        <v>57.31949579831938</v>
       </c>
     </row>
     <row r="155">
@@ -8527,7 +8572,7 @@
         </is>
       </c>
       <c r="H155">
-        <v>-2.749999999999964</v>
+        <v>-3.236234380593075</v>
       </c>
       <c r="I155">
         <v>2023</v>
@@ -8552,7 +8597,7 @@
         <v>2015</v>
       </c>
       <c r="O155">
-        <v>82.00000000000014</v>
+        <v>81.52250836120407</v>
       </c>
     </row>
     <row r="156">
@@ -8581,7 +8626,7 @@
         </is>
       </c>
       <c r="H156">
-        <v>0.40625</v>
+        <v>0.4166666666666998</v>
       </c>
       <c r="I156">
         <v>2023</v>
@@ -8606,7 +8651,7 @@
         <v>2015</v>
       </c>
       <c r="O156">
-        <v>70.60000000000001</v>
+        <v>70.50153846153836</v>
       </c>
     </row>
     <row r="157">
@@ -8635,7 +8680,7 @@
         </is>
       </c>
       <c r="H157">
-        <v>-1.770833333333361</v>
+        <v>-2.056590656284733</v>
       </c>
       <c r="I157">
         <v>2023</v>
@@ -8660,7 +8705,7 @@
         <v>2015</v>
       </c>
       <c r="O157">
-        <v>51.1</v>
+        <v>50.40838709677425</v>
       </c>
     </row>
     <row r="158">
@@ -8689,7 +8734,7 @@
         </is>
       </c>
       <c r="H158">
-        <v>2.12500000000006</v>
+        <v>2.255233990147822</v>
       </c>
       <c r="I158">
         <v>2023</v>
@@ -8714,7 +8759,7 @@
         <v>2015</v>
       </c>
       <c r="O158">
-        <v>39.79999999999993</v>
+        <v>39.63999999999999</v>
       </c>
     </row>
     <row r="159">
@@ -8743,7 +8788,7 @@
         </is>
       </c>
       <c r="H159">
-        <v>1.25</v>
+        <v>1.554966266135338</v>
       </c>
       <c r="I159">
         <v>2023</v>
@@ -8768,7 +8813,7 @@
         <v>2015</v>
       </c>
       <c r="O159">
-        <v>77</v>
+        <v>76.45747676343261</v>
       </c>
     </row>
     <row r="160">
@@ -8797,7 +8842,7 @@
         </is>
       </c>
       <c r="H160">
-        <v>-2.1875</v>
+        <v>-4.138777888777881</v>
       </c>
       <c r="I160">
         <v>2023</v>
@@ -8822,7 +8867,7 @@
         <v>2015</v>
       </c>
       <c r="O160">
-        <v>90.10000000000001</v>
+        <v>89.78500000000001</v>
       </c>
     </row>
     <row r="161">
@@ -8851,7 +8896,7 @@
         </is>
       </c>
       <c r="H161">
-        <v>-3.208333333333194</v>
+        <v>-4.244778522600647</v>
       </c>
       <c r="I161">
         <v>2023</v>
@@ -8876,7 +8921,7 @@
         <v>2015</v>
       </c>
       <c r="O161">
-        <v>85.80000000000001</v>
+        <v>85.28455882352944</v>
       </c>
     </row>
     <row r="162">
@@ -8905,7 +8950,7 @@
         </is>
       </c>
       <c r="H162">
-        <v>-1.6875</v>
+        <v>-1.771938942991561</v>
       </c>
       <c r="I162">
         <v>2023</v>
@@ -8930,7 +8975,7 @@
         <v>2015</v>
       </c>
       <c r="O162">
-        <v>66.5</v>
+        <v>66.48717948717949</v>
       </c>
     </row>
     <row r="163">
@@ -8959,7 +9004,7 @@
         </is>
       </c>
       <c r="H163">
-        <v>0.75</v>
+        <v>1.250000000000014</v>
       </c>
       <c r="I163">
         <v>2023</v>
@@ -8984,7 +9029,7 @@
         <v>2015</v>
       </c>
       <c r="O163">
-        <v>90.90000000000001</v>
+        <v>90.58</v>
       </c>
     </row>
     <row r="164">
@@ -9013,7 +9058,7 @@
         </is>
       </c>
       <c r="H164">
-        <v>1.604166666666579</v>
+        <v>2.444140736611509</v>
       </c>
       <c r="I164">
         <v>2023</v>
@@ -9038,7 +9083,7 @@
         <v>2015</v>
       </c>
       <c r="O164">
-        <v>83.30000000000015</v>
+        <v>82.63448146056845</v>
       </c>
     </row>
     <row r="165">
@@ -9067,7 +9112,7 @@
         </is>
       </c>
       <c r="H165">
-        <v>-3.03125</v>
+        <v>-3.426059932147318</v>
       </c>
       <c r="I165">
         <v>2023</v>
@@ -9092,7 +9137,7 @@
         <v>2015</v>
       </c>
       <c r="O165">
-        <v>80.05000000000011</v>
+        <v>79.71333880678711</v>
       </c>
     </row>
     <row r="166">
@@ -9121,7 +9166,7 @@
         </is>
       </c>
       <c r="H166">
-        <v>3.708333333333272</v>
+        <v>6.172177871578022</v>
       </c>
       <c r="I166">
         <v>2023</v>
@@ -9146,7 +9191,7 @@
         <v>2015</v>
       </c>
       <c r="O166">
-        <v>84.40000000000015</v>
+        <v>83.57345864661653</v>
       </c>
     </row>
     <row r="167">
@@ -9175,7 +9220,7 @@
         </is>
       </c>
       <c r="H167">
-        <v>-1.8125</v>
+        <v>-3.159722222222243</v>
       </c>
       <c r="I167">
         <v>2023</v>
@@ -9200,7 +9245,7 @@
         <v>2015</v>
       </c>
       <c r="O167">
-        <v>91.30000000000001</v>
+        <v>90.93333333333332</v>
       </c>
     </row>
     <row r="168">
@@ -9229,7 +9274,7 @@
         </is>
       </c>
       <c r="H168">
-        <v>-0.625</v>
+        <v>-0.892857142857153</v>
       </c>
       <c r="I168">
         <v>2023</v>
@@ -9254,7 +9299,7 @@
         <v>2015</v>
       </c>
       <c r="O168">
-        <v>90.7</v>
+        <v>90.40857142857143</v>
       </c>
     </row>
     <row r="169">
@@ -9283,7 +9328,7 @@
         </is>
       </c>
       <c r="H169">
-        <v>4.875000000000004</v>
+        <v>5.418763944136451</v>
       </c>
       <c r="I169">
         <v>2023</v>
@@ -9308,7 +9353,7 @@
         <v>2015</v>
       </c>
       <c r="O169">
-        <v>53</v>
+        <v>52.386875</v>
       </c>
     </row>
     <row r="170">
@@ -9337,7 +9382,7 @@
         </is>
       </c>
       <c r="H170">
-        <v>-0.2083333333333215</v>
+        <v>-0.224867724867714</v>
       </c>
       <c r="I170">
         <v>2023</v>
@@ -9362,7 +9407,7 @@
         <v>2015</v>
       </c>
       <c r="O170">
-        <v>81.20000000000014</v>
+        <v>80.83401709401714</v>
       </c>
     </row>
     <row r="171">
@@ -9391,7 +9436,7 @@
         </is>
       </c>
       <c r="H171">
-        <v>0.125</v>
+        <v>0.1470588235294201</v>
       </c>
       <c r="I171">
         <v>2023</v>
@@ -9416,7 +9461,7 @@
         <v>2015</v>
       </c>
       <c r="O171">
-        <v>77.60000000000001</v>
+        <v>76.99411541889479</v>
       </c>
     </row>
     <row r="172">
@@ -9445,7 +9490,7 @@
         </is>
       </c>
       <c r="H172">
-        <v>1</v>
+        <v>1.017628205128261</v>
       </c>
       <c r="I172">
         <v>2023</v>
@@ -9470,7 +9515,7 @@
         <v>2015</v>
       </c>
       <c r="O172">
-        <v>69.60000000000001</v>
+        <v>69.54499999999986</v>
       </c>
     </row>
     <row r="173">
@@ -9499,7 +9544,7 @@
         </is>
       </c>
       <c r="H173">
-        <v>1.625</v>
+        <v>1.880777954989284</v>
       </c>
       <c r="I173">
         <v>2023</v>
@@ -9524,7 +9569,7 @@
         <v>2015</v>
       </c>
       <c r="O173">
-        <v>74.5</v>
+        <v>74.18183183183194</v>
       </c>
     </row>
     <row r="174">
@@ -9553,7 +9598,7 @@
         </is>
       </c>
       <c r="H174">
-        <v>1.3125</v>
+        <v>1.491013071895409</v>
       </c>
       <c r="I174">
         <v>2023</v>
@@ -9578,7 +9623,7 @@
         <v>2015</v>
       </c>
       <c r="O174">
-        <v>17.5</v>
+        <v>17.2929411764706</v>
       </c>
     </row>
     <row r="175">
@@ -9607,7 +9652,7 @@
         </is>
       </c>
       <c r="H175">
-        <v>-2.270833333333286</v>
+        <v>-3.460597784997937</v>
       </c>
       <c r="I175">
         <v>2023</v>
@@ -9632,7 +9677,7 @@
         <v>2015</v>
       </c>
       <c r="O175">
-        <v>88.5</v>
+        <v>87.78787878787878</v>
       </c>
     </row>
     <row r="176">
@@ -9661,7 +9706,7 @@
         </is>
       </c>
       <c r="H176">
-        <v>3.249999999999964</v>
+        <v>3.762595762217579</v>
       </c>
       <c r="I176">
         <v>2023</v>
@@ -9686,7 +9731,7 @@
         <v>2015</v>
       </c>
       <c r="O176">
-        <v>72.90000000000001</v>
+        <v>72.69110624794848</v>
       </c>
     </row>
     <row r="177">
@@ -9715,7 +9760,7 @@
         </is>
       </c>
       <c r="H177">
-        <v>-3.1145833333333</v>
+        <v>-3.616678083405169</v>
       </c>
       <c r="I177">
         <v>2023</v>
@@ -9740,7 +9785,7 @@
         <v>2015</v>
       </c>
       <c r="O177">
-        <v>81.90000000000015</v>
+        <v>81.43789297658867</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update and run scripts
</commit_message>
<xml_diff>
--- a/intermediate/dashboard_output_gender.xlsx
+++ b/intermediate/dashboard_output_gender.xlsx
@@ -457,13 +457,13 @@
         </is>
       </c>
       <c r="H2">
-        <v>-36.80769233684551</v>
+        <v>-37.95833333333369</v>
       </c>
       <c r="I2">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="J2">
-        <v>2.6</v>
+        <v>6.5</v>
       </c>
       <c r="K2">
         <v>53.3</v>
@@ -482,7 +482,7 @@
         <v>2015</v>
       </c>
       <c r="O2">
-        <v>56.05588235294112</v>
+        <v>55.7</v>
       </c>
     </row>
     <row r="3">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="H3">
-        <v>1.875658004914925</v>
+        <v>1.637499999999989</v>
       </c>
       <c r="I3">
         <v>2023</v>
@@ -536,7 +536,7 @@
         <v>2015</v>
       </c>
       <c r="O3">
-        <v>72.87815078236147</v>
+        <v>73.26000000000003</v>
       </c>
     </row>
     <row r="4">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="H4">
-        <v>7.67750368611437</v>
+        <v>4.958333333333307</v>
       </c>
       <c r="I4">
         <v>2023</v>
@@ -590,7 +590,7 @@
         <v>2015</v>
       </c>
       <c r="O4">
-        <v>84.51233574131409</v>
+        <v>85.06666666666671</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="H5">
-        <v>5.470000115780927</v>
+        <v>5.08333333333341</v>
       </c>
       <c r="I5">
         <v>2023</v>
@@ -644,7 +644,7 @@
         <v>2015</v>
       </c>
       <c r="O5">
-        <v>46.06896551724144</v>
+        <v>46.09999999999993</v>
       </c>
     </row>
     <row r="6">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="H6">
-        <v>1.501528496013805</v>
+        <v>1.125</v>
       </c>
       <c r="I6">
         <v>2023</v>
@@ -698,7 +698,7 @@
         <v>2015</v>
       </c>
       <c r="O6">
-        <v>85.54598039215685</v>
+        <v>85.90000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="H7">
-        <v>9.850563668826972</v>
+        <v>6.656249999999879</v>
       </c>
       <c r="I7">
         <v>2023</v>
@@ -752,7 +752,7 @@
         <v>2015</v>
       </c>
       <c r="O7">
-        <v>77.52371700879768</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="8">
@@ -780,18 +780,12 @@
           <t>AUS</t>
         </is>
       </c>
-      <c r="H8">
-        <v>-9.166666666666657</v>
-      </c>
       <c r="I8">
         <v>2023</v>
       </c>
       <c r="J8">
         <v>91.7</v>
       </c>
-      <c r="K8">
-        <v>93.60000000000001</v>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>45.0.0</t>
@@ -801,12 +795,6 @@
         <is>
           <t>Women political empowerment index</t>
         </is>
-      </c>
-      <c r="N8">
-        <v>2015</v>
-      </c>
-      <c r="O8">
-        <v>93.68000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -877,7 +865,7 @@
         </is>
       </c>
       <c r="H10">
-        <v>0.0625</v>
+        <v>0.04999999999999716</v>
       </c>
       <c r="I10">
         <v>2023</v>
@@ -902,7 +890,7 @@
         <v>2015</v>
       </c>
       <c r="O10">
-        <v>69.15499999999989</v>
+        <v>70.00000000000023</v>
       </c>
     </row>
     <row r="11">
@@ -931,7 +919,7 @@
         </is>
       </c>
       <c r="H11">
-        <v>2.645748987854283</v>
+        <v>2.33124999999994</v>
       </c>
       <c r="I11">
         <v>2023</v>
@@ -956,7 +944,7 @@
         <v>2015</v>
       </c>
       <c r="O11">
-        <v>62.57526315789475</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="12">
@@ -1027,7 +1015,7 @@
         </is>
       </c>
       <c r="H13">
-        <v>3.86207970950619</v>
+        <v>2.499999999999993</v>
       </c>
       <c r="I13">
         <v>2023</v>
@@ -1052,7 +1040,7 @@
         <v>2015</v>
       </c>
       <c r="O13">
-        <v>85.19632352941177</v>
+        <v>85.60000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1081,7 +1069,7 @@
         </is>
       </c>
       <c r="H14">
-        <v>-1.89182437208752</v>
+        <v>-1.599999999999959</v>
       </c>
       <c r="I14">
         <v>2023</v>
@@ -1106,7 +1094,7 @@
         <v>2015</v>
       </c>
       <c r="O14">
-        <v>76.18827094474153</v>
+        <v>76.7</v>
       </c>
     </row>
     <row r="15">
@@ -1135,7 +1123,7 @@
         </is>
       </c>
       <c r="H15">
-        <v>-0.1282051282051384</v>
+        <v>-0.09999999999999432</v>
       </c>
       <c r="I15">
         <v>2023</v>
@@ -1160,7 +1148,7 @@
         <v>2015</v>
       </c>
       <c r="O15">
-        <v>72.69110624794848</v>
+        <v>73.10000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -1189,7 +1177,7 @@
         </is>
       </c>
       <c r="H16">
-        <v>0.9583333333333357</v>
+        <v>0.5</v>
       </c>
       <c r="I16">
         <v>2023</v>
@@ -1214,7 +1202,7 @@
         <v>2015</v>
       </c>
       <c r="O16">
-        <v>91.01666666666667</v>
+        <v>91.40000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1243,7 +1231,7 @@
         </is>
       </c>
       <c r="H17">
-        <v>5.244904330340312</v>
+        <v>4.875000000000075</v>
       </c>
       <c r="I17">
         <v>2023</v>
@@ -1268,7 +1256,7 @@
         <v>2015</v>
       </c>
       <c r="O17">
-        <v>46.27586206896555</v>
+        <v>46.29999999999993</v>
       </c>
     </row>
     <row r="18">
@@ -1297,7 +1285,7 @@
         </is>
       </c>
       <c r="H18">
-        <v>-2.289352363752513</v>
+        <v>-1.583333333333279</v>
       </c>
       <c r="I18">
         <v>2023</v>
@@ -1322,7 +1310,7 @@
         <v>2015</v>
       </c>
       <c r="O18">
-        <v>86.31571428571428</v>
+        <v>86.80000000000001</v>
       </c>
     </row>
     <row r="19">
@@ -1351,7 +1339,7 @@
         </is>
       </c>
       <c r="H19">
-        <v>-5.585035079768971</v>
+        <v>-4.218749999999879</v>
       </c>
       <c r="I19">
         <v>2023</v>
@@ -1376,7 +1364,7 @@
         <v>2015</v>
       </c>
       <c r="O19">
-        <v>85.4610294117647</v>
+        <v>85.80000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1405,7 +1393,7 @@
         </is>
       </c>
       <c r="H20">
-        <v>2.553444710110277</v>
+        <v>1.968749999999936</v>
       </c>
       <c r="I20">
         <v>2023</v>
@@ -1430,7 +1418,7 @@
         <v>2015</v>
       </c>
       <c r="O20">
-        <v>78.75665580804073</v>
+        <v>79.47500000000002</v>
       </c>
     </row>
     <row r="21">
@@ -1459,7 +1447,7 @@
         </is>
       </c>
       <c r="H21">
-        <v>-0.7594285243741652</v>
+        <v>-0.5833333333333002</v>
       </c>
       <c r="I21">
         <v>2023</v>
@@ -1484,7 +1472,7 @@
         <v>2015</v>
       </c>
       <c r="O21">
-        <v>83.40592617908406</v>
+        <v>84.20000000000009</v>
       </c>
     </row>
     <row r="22">
@@ -1513,7 +1501,7 @@
         </is>
       </c>
       <c r="H22">
-        <v>4.176136363636367</v>
+        <v>2.625</v>
       </c>
       <c r="I22">
         <v>2023</v>
@@ -1538,7 +1526,7 @@
         <v>2015</v>
       </c>
       <c r="O22">
-        <v>88.38818181818182</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23">
@@ -1567,7 +1555,7 @@
         </is>
       </c>
       <c r="H23">
-        <v>0.04032258064516014</v>
+        <v>0.03125</v>
       </c>
       <c r="I23">
         <v>2023</v>
@@ -1592,7 +1580,7 @@
         <v>2015</v>
       </c>
       <c r="O23">
-        <v>79.01794613062134</v>
+        <v>79.7</v>
       </c>
     </row>
     <row r="24">
@@ -1621,7 +1609,7 @@
         </is>
       </c>
       <c r="H24">
-        <v>-1.491123808461232</v>
+        <v>-1.331249999999997</v>
       </c>
       <c r="I24">
         <v>2023</v>
@@ -1646,7 +1634,7 @@
         <v>2015</v>
       </c>
       <c r="O24">
-        <v>77.34724642056237</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25">
@@ -1675,7 +1663,7 @@
         </is>
       </c>
       <c r="H25">
-        <v>-0.9836506547032542</v>
+        <v>-0.9375</v>
       </c>
       <c r="I25">
         <v>2023</v>
@@ -1700,7 +1688,7 @@
         <v>2015</v>
       </c>
       <c r="O25">
-        <v>65.15384615384602</v>
+        <v>65.60000000000012</v>
       </c>
     </row>
     <row r="26">
@@ -1729,7 +1717,7 @@
         </is>
       </c>
       <c r="H26">
-        <v>-6.281250000000028</v>
+        <v>-3.5</v>
       </c>
       <c r="I26">
         <v>2023</v>
@@ -1754,7 +1742,7 @@
         <v>2015</v>
       </c>
       <c r="O26">
-        <v>92.19000000000001</v>
+        <v>92.7</v>
       </c>
     </row>
     <row r="27">
@@ -1782,17 +1770,11 @@
           <t>CHE</t>
         </is>
       </c>
-      <c r="H27">
-        <v>5</v>
-      </c>
       <c r="I27">
         <v>2023</v>
       </c>
       <c r="J27">
-        <v>94.2</v>
-      </c>
-      <c r="K27">
-        <v>93.80000000000001</v>
+        <v>94.19999999999999</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1803,12 +1785,6 @@
         <is>
           <t>Women political empowerment index</t>
         </is>
-      </c>
-      <c r="N27">
-        <v>2015</v>
-      </c>
-      <c r="O27">
-        <v>93.88000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1837,7 +1813,7 @@
         </is>
       </c>
       <c r="H28">
-        <v>7.70265151515153</v>
+        <v>4.5625</v>
       </c>
       <c r="I28">
         <v>2023</v>
@@ -1862,7 +1838,7 @@
         <v>2015</v>
       </c>
       <c r="O28">
-        <v>87.43000000000001</v>
+        <v>88.10000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1891,7 +1867,7 @@
         </is>
       </c>
       <c r="H29">
-        <v>-1.700906371959</v>
+        <v>-1.625</v>
       </c>
       <c r="I29">
         <v>2023</v>
@@ -1916,7 +1892,7 @@
         <v>2015</v>
       </c>
       <c r="O29">
-        <v>66.69230769230762</v>
+        <v>67.47500000000025</v>
       </c>
     </row>
     <row r="30">
@@ -1945,7 +1921,7 @@
         </is>
       </c>
       <c r="H30">
-        <v>0.5904639457270733</v>
+        <v>0.4874999999999829</v>
       </c>
       <c r="I30">
         <v>2023</v>
@@ -1970,7 +1946,7 @@
         <v>2015</v>
       </c>
       <c r="O30">
-        <v>72.50649086333311</v>
+        <v>72.94000000000005</v>
       </c>
     </row>
     <row r="31">
@@ -1999,7 +1975,7 @@
         </is>
       </c>
       <c r="H31">
-        <v>0.2831196581196522</v>
+        <v>0.2395833333333215</v>
       </c>
       <c r="I31">
         <v>2023</v>
@@ -2024,7 +2000,7 @@
         <v>2015</v>
       </c>
       <c r="O31">
-        <v>81.00713675213679</v>
+        <v>81.42500000000013</v>
       </c>
     </row>
     <row r="32">
@@ -2053,7 +2029,7 @@
         </is>
       </c>
       <c r="H32">
-        <v>0.9403548351158975</v>
+        <v>0.78125</v>
       </c>
       <c r="I32">
         <v>2023</v>
@@ -2078,7 +2054,7 @@
         <v>2015</v>
       </c>
       <c r="O32">
-        <v>54.06223484848478</v>
+        <v>54.6</v>
       </c>
     </row>
     <row r="33">
@@ -2107,7 +2083,7 @@
         </is>
       </c>
       <c r="H33">
-        <v>4.741686314962283</v>
+        <v>4.375000000000124</v>
       </c>
       <c r="I33">
         <v>2023</v>
@@ -2132,7 +2108,7 @@
         <v>2015</v>
       </c>
       <c r="O33">
-        <v>34.63692307692303</v>
+        <v>34.89999999999993</v>
       </c>
     </row>
     <row r="34">
@@ -2161,7 +2137,7 @@
         </is>
       </c>
       <c r="H34">
-        <v>0.4185744810744794</v>
+        <v>0.3229166666666572</v>
       </c>
       <c r="I34">
         <v>2023</v>
@@ -2186,7 +2162,7 @@
         <v>2015</v>
       </c>
       <c r="O34">
-        <v>80.65941391941395</v>
+        <v>81.12500000000013</v>
       </c>
     </row>
     <row r="35">
@@ -2215,7 +2191,7 @@
         </is>
       </c>
       <c r="H35">
-        <v>1.073626893939412</v>
+        <v>0.875</v>
       </c>
       <c r="I35">
         <v>2023</v>
@@ -2240,7 +2216,7 @@
         <v>2015</v>
       </c>
       <c r="O35">
-        <v>53.00562499999994</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="36">
@@ -2269,7 +2245,7 @@
         </is>
       </c>
       <c r="H36">
-        <v>1.349611367846478</v>
+        <v>0.9583333333332789</v>
       </c>
       <c r="I36">
         <v>2023</v>
@@ -2294,7 +2270,7 @@
         <v>2015</v>
       </c>
       <c r="O36">
-        <v>82.55114812723514</v>
+        <v>83.20000000000014</v>
       </c>
     </row>
     <row r="37">
@@ -2323,7 +2299,7 @@
         </is>
       </c>
       <c r="H37">
-        <v>-1.041666666666664</v>
+        <v>-0.375</v>
       </c>
       <c r="I37">
         <v>2023</v>
@@ -2348,7 +2324,7 @@
         <v>2015</v>
       </c>
       <c r="O37">
-        <v>92.44000000000001</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38">
@@ -2377,7 +2353,7 @@
         </is>
       </c>
       <c r="H38">
-        <v>0.739709851552</v>
+        <v>0.5749999999999673</v>
       </c>
       <c r="I38">
         <v>2023</v>
@@ -2402,7 +2378,7 @@
         <v>2015</v>
       </c>
       <c r="O38">
-        <v>70.891282051282</v>
+        <v>71.58000000000011</v>
       </c>
     </row>
     <row r="39">
@@ -2431,7 +2407,7 @@
         </is>
       </c>
       <c r="H39">
-        <v>-0.3229166666666714</v>
+        <v>-0.25</v>
       </c>
       <c r="I39">
         <v>2023</v>
@@ -2456,7 +2432,7 @@
         <v>2015</v>
       </c>
       <c r="O39">
-        <v>86.31571428571428</v>
+        <v>86.80000000000001</v>
       </c>
     </row>
     <row r="40">
@@ -2485,7 +2461,7 @@
         </is>
       </c>
       <c r="H40">
-        <v>8.229166666666657</v>
+        <v>2.375</v>
       </c>
       <c r="I40">
         <v>2023</v>
@@ -2510,7 +2486,7 @@
         <v>2015</v>
       </c>
       <c r="O40">
-        <v>91.72</v>
+        <v>92.2</v>
       </c>
     </row>
     <row r="41">
@@ -2581,7 +2557,7 @@
         </is>
       </c>
       <c r="H42">
-        <v>2.534207026273563</v>
+        <v>2.25</v>
       </c>
       <c r="I42">
         <v>2023</v>
@@ -2606,7 +2582,7 @@
         <v>2015</v>
       </c>
       <c r="O42">
-        <v>55.52869875222807</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43">
@@ -2677,7 +2653,7 @@
         </is>
       </c>
       <c r="H44">
-        <v>1.585356981881574</v>
+        <v>1.124999999999936</v>
       </c>
       <c r="I44">
         <v>2023</v>
@@ -2702,7 +2678,7 @@
         <v>2015</v>
       </c>
       <c r="O44">
-        <v>82.38370553359687</v>
+        <v>83.00000000000014</v>
       </c>
     </row>
     <row r="45">
@@ -2731,7 +2707,7 @@
         </is>
       </c>
       <c r="H45">
-        <v>-5.213858340635426</v>
+        <v>-4.306249999999899</v>
       </c>
       <c r="I45">
         <v>2023</v>
@@ -2756,7 +2732,7 @@
         <v>2015</v>
       </c>
       <c r="O45">
-        <v>80.14483284914326</v>
+        <v>80.67500000000008</v>
       </c>
     </row>
     <row r="46">
@@ -2785,7 +2761,7 @@
         </is>
       </c>
       <c r="H46">
-        <v>-3.366025690425843</v>
+        <v>-2.3541666666666</v>
       </c>
       <c r="I46">
         <v>2023</v>
@@ -2810,7 +2786,7 @@
         <v>2015</v>
       </c>
       <c r="O46">
-        <v>87.09076923076927</v>
+        <v>87.7</v>
       </c>
     </row>
     <row r="47">
@@ -2839,7 +2815,7 @@
         </is>
       </c>
       <c r="H47">
-        <v>10.99685073961445</v>
+        <v>10.15625000000023</v>
       </c>
       <c r="I47">
         <v>2023</v>
@@ -2864,7 +2840,7 @@
         <v>2015</v>
       </c>
       <c r="O47">
-        <v>32.78</v>
+        <v>33.09999999999993</v>
       </c>
     </row>
     <row r="48">
@@ -2893,7 +2869,7 @@
         </is>
       </c>
       <c r="H48">
-        <v>1.352339181286517</v>
+        <v>1.25</v>
       </c>
       <c r="I48">
         <v>2023</v>
@@ -2918,7 +2894,7 @@
         <v>2015</v>
       </c>
       <c r="O48">
-        <v>18.46444444444448</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="49">
@@ -3031,7 +3007,7 @@
         </is>
       </c>
       <c r="H51">
-        <v>1.695853676116812</v>
+        <v>1.443749999999966</v>
       </c>
       <c r="I51">
         <v>2023</v>
@@ -3056,7 +3032,7 @@
         <v>2015</v>
       </c>
       <c r="O51">
-        <v>71.37376518218628</v>
+        <v>71.9800000000001</v>
       </c>
     </row>
     <row r="52">
@@ -3127,7 +3103,7 @@
         </is>
       </c>
       <c r="H53">
-        <v>-1.496204453441344</v>
+        <v>-1.174999999999933</v>
       </c>
       <c r="I53">
         <v>2023</v>
@@ -3152,7 +3128,7 @@
         <v>2015</v>
       </c>
       <c r="O53">
-        <v>73.2570981507825</v>
+        <v>73.58000000000003</v>
       </c>
     </row>
     <row r="54">
@@ -3180,18 +3156,12 @@
           <t>FRA</t>
         </is>
       </c>
-      <c r="H54">
-        <v>-8.75</v>
-      </c>
       <c r="I54">
         <v>2023</v>
       </c>
       <c r="J54">
         <v>93</v>
       </c>
-      <c r="K54">
-        <v>94</v>
-      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>45.0.0</t>
@@ -3201,12 +3171,6 @@
         <is>
           <t>Women political empowerment index</t>
         </is>
-      </c>
-      <c r="N54">
-        <v>2015</v>
-      </c>
-      <c r="O54">
-        <v>94.08000000000001</v>
       </c>
     </row>
     <row r="55">
@@ -3235,7 +3199,7 @@
         </is>
       </c>
       <c r="H55">
-        <v>2.28651679668431</v>
+        <v>1.781249999999964</v>
       </c>
       <c r="I55">
         <v>2023</v>
@@ -3260,7 +3224,7 @@
         <v>2015</v>
       </c>
       <c r="O55">
-        <v>77.87777492668626</v>
+        <v>78.60000000000001</v>
       </c>
     </row>
     <row r="56">
@@ -3289,7 +3253,7 @@
         </is>
       </c>
       <c r="H56">
-        <v>0.625</v>
+        <v>0.25</v>
       </c>
       <c r="I56">
         <v>2023</v>
@@ -3314,7 +3278,7 @@
         <v>2015</v>
       </c>
       <c r="O56">
-        <v>91.82000000000001</v>
+        <v>92.30000000000001</v>
       </c>
     </row>
     <row r="57">
@@ -3343,7 +3307,7 @@
         </is>
       </c>
       <c r="H57">
-        <v>6.115003686114356</v>
+        <v>3.833333333333307</v>
       </c>
       <c r="I57">
         <v>2023</v>
@@ -3368,7 +3332,7 @@
         <v>2015</v>
       </c>
       <c r="O57">
-        <v>84.51233574131409</v>
+        <v>85.06666666666671</v>
       </c>
     </row>
     <row r="58">
@@ -3397,7 +3361,7 @@
         </is>
       </c>
       <c r="H58">
-        <v>2.312400953991315</v>
+        <v>1.749999999999908</v>
       </c>
       <c r="I58">
         <v>2023</v>
@@ -3422,7 +3386,7 @@
         <v>2015</v>
       </c>
       <c r="O58">
-        <v>80.74512820512822</v>
+        <v>81.20000000000014</v>
       </c>
     </row>
     <row r="59">
@@ -3451,7 +3415,7 @@
         </is>
       </c>
       <c r="H59">
-        <v>1.185735887096762</v>
+        <v>1.125000000000021</v>
       </c>
       <c r="I59">
         <v>2023</v>
@@ -3476,7 +3440,7 @@
         <v>2015</v>
       </c>
       <c r="O59">
-        <v>50.92451612903228</v>
+        <v>50.99999999999991</v>
       </c>
     </row>
     <row r="60">
@@ -3505,7 +3469,7 @@
         </is>
       </c>
       <c r="H60">
-        <v>8.954765375439841</v>
+        <v>7.608333333333199</v>
       </c>
       <c r="I60">
         <v>2023</v>
@@ -3530,7 +3494,7 @@
         <v>2015</v>
       </c>
       <c r="O60">
-        <v>58.05547619047624</v>
+        <v>58.40000000000001</v>
       </c>
     </row>
     <row r="61">
@@ -3559,7 +3523,7 @@
         </is>
       </c>
       <c r="H61">
-        <v>-4.151817303133122</v>
+        <v>-3.587499999999899</v>
       </c>
       <c r="I61">
         <v>2023</v>
@@ -3584,7 +3548,7 @@
         <v>2015</v>
       </c>
       <c r="O61">
-        <v>74.54991848991855</v>
+        <v>74.90000000000001</v>
       </c>
     </row>
     <row r="62">
@@ -3613,7 +3577,7 @@
         </is>
       </c>
       <c r="H62">
-        <v>1.169813049853374</v>
+        <v>1.052083333333346</v>
       </c>
       <c r="I62">
         <v>2023</v>
@@ -3638,7 +3602,7 @@
         <v>2015</v>
       </c>
       <c r="O62">
-        <v>51.65169354838709</v>
+        <v>51.93333333333331</v>
       </c>
     </row>
     <row r="63">
@@ -3667,7 +3631,7 @@
         </is>
       </c>
       <c r="H63">
-        <v>-6.645833333333321</v>
+        <v>-2.625</v>
       </c>
       <c r="I63">
         <v>2023</v>
@@ -3692,7 +3656,7 @@
         <v>2015</v>
       </c>
       <c r="O63">
-        <v>92.89333333333333</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="64">
@@ -3721,7 +3685,7 @@
         </is>
       </c>
       <c r="H64">
-        <v>1.64945562971878</v>
+        <v>1.38749999999996</v>
       </c>
       <c r="I64">
         <v>2023</v>
@@ -3746,7 +3710,7 @@
         <v>2015</v>
       </c>
       <c r="O64">
-        <v>70.98871794871793</v>
+        <v>71.66000000000014</v>
       </c>
     </row>
     <row r="65">
@@ -3775,7 +3739,7 @@
         </is>
       </c>
       <c r="H65">
-        <v>-2.927671287046309</v>
+        <v>-1.9375</v>
       </c>
       <c r="I65">
         <v>2023</v>
@@ -3800,7 +3764,7 @@
         <v>2015</v>
       </c>
       <c r="O65">
-        <v>88.38818181818182</v>
+        <v>89</v>
       </c>
     </row>
     <row r="66">
@@ -3829,7 +3793,7 @@
         </is>
       </c>
       <c r="H66">
-        <v>-9.853654909033331</v>
+        <v>-6.374999999999929</v>
       </c>
       <c r="I66">
         <v>2023</v>
@@ -3854,7 +3818,7 @@
         <v>2015</v>
       </c>
       <c r="O66">
-        <v>91.01666666666667</v>
+        <v>91.40000000000001</v>
       </c>
     </row>
     <row r="67">
@@ -3883,7 +3847,7 @@
         </is>
       </c>
       <c r="H67">
-        <v>2.797328166686867</v>
+        <v>2.229166666666643</v>
       </c>
       <c r="I67">
         <v>2023</v>
@@ -3908,7 +3872,7 @@
         <v>2015</v>
       </c>
       <c r="O67">
-        <v>76.00541380188436</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="68">
@@ -3937,7 +3901,7 @@
         </is>
       </c>
       <c r="H68">
-        <v>8.104166666666686</v>
+        <v>3.875</v>
       </c>
       <c r="I68">
         <v>2023</v>
@@ -3962,7 +3926,7 @@
         <v>2015</v>
       </c>
       <c r="O68">
-        <v>89.95999999999999</v>
+        <v>90.2</v>
       </c>
     </row>
     <row r="69">
@@ -3991,7 +3955,7 @@
         </is>
       </c>
       <c r="H69">
-        <v>-5.592150505943728</v>
+        <v>-5.125000000000146</v>
       </c>
       <c r="I69">
         <v>2023</v>
@@ -4016,7 +3980,7 @@
         <v>2015</v>
       </c>
       <c r="O69">
-        <v>45.65517241379311</v>
+        <v>45.69999999999993</v>
       </c>
     </row>
     <row r="70">
@@ -4070,7 +4034,7 @@
         <v>2015</v>
       </c>
       <c r="O70">
-        <v>86.56989010989011</v>
+        <v>87.10000000000001</v>
       </c>
     </row>
     <row r="71">
@@ -4099,7 +4063,7 @@
         </is>
       </c>
       <c r="H71">
-        <v>-1.589626569889674</v>
+        <v>-1.38124999999998</v>
       </c>
       <c r="I71">
         <v>2023</v>
@@ -4124,7 +4088,7 @@
         <v>2015</v>
       </c>
       <c r="O71">
-        <v>76.63461962057546</v>
+        <v>77.2</v>
       </c>
     </row>
     <row r="72">
@@ -4153,7 +4117,7 @@
         </is>
       </c>
       <c r="H72">
-        <v>-0.59375</v>
+        <v>-0.474999999999973</v>
       </c>
       <c r="I72">
         <v>2023</v>
@@ -4178,7 +4142,7 @@
         <v>2015</v>
       </c>
       <c r="O72">
-        <v>70.21653846153831</v>
+        <v>71.02000000000017</v>
       </c>
     </row>
     <row r="73">
@@ -4207,7 +4171,7 @@
         </is>
       </c>
       <c r="H73">
-        <v>6.979166666666657</v>
+        <v>2.5</v>
       </c>
       <c r="I73">
         <v>2023</v>
@@ -4232,7 +4196,7 @@
         <v>2015</v>
       </c>
       <c r="O73">
-        <v>91.30000000000001</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="74">
@@ -4261,7 +4225,7 @@
         </is>
       </c>
       <c r="H74">
-        <v>-1.205484330484364</v>
+        <v>-1.083333333333364</v>
       </c>
       <c r="I74">
         <v>2023</v>
@@ -4286,7 +4250,7 @@
         <v>2015</v>
       </c>
       <c r="O74">
-        <v>37.79185185185178</v>
+        <v>37.99999999999993</v>
       </c>
     </row>
     <row r="75">
@@ -4315,7 +4279,7 @@
         </is>
       </c>
       <c r="H75">
-        <v>0.4569128787878896</v>
+        <v>0.375</v>
       </c>
       <c r="I75">
         <v>2023</v>
@@ -4340,7 +4304,7 @@
         <v>2015</v>
       </c>
       <c r="O75">
-        <v>53.95598484848477</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="76">
@@ -4369,7 +4333,7 @@
         </is>
       </c>
       <c r="H76">
-        <v>-9.180555555555571</v>
+        <v>-4.6875</v>
       </c>
       <c r="I76">
         <v>2023</v>
@@ -4394,7 +4358,7 @@
         <v>2015</v>
       </c>
       <c r="O76">
-        <v>92.74000000000001</v>
+        <v>93.30000000000001</v>
       </c>
     </row>
     <row r="77">
@@ -4423,7 +4387,7 @@
         </is>
       </c>
       <c r="H77">
-        <v>-0.6388888888888857</v>
+        <v>-0.3125</v>
       </c>
       <c r="I77">
         <v>2023</v>
@@ -4448,7 +4412,7 @@
         <v>2015</v>
       </c>
       <c r="O77">
-        <v>88.99555555555557</v>
+        <v>89.35000000000001</v>
       </c>
     </row>
     <row r="78">
@@ -4477,7 +4441,7 @@
         </is>
       </c>
       <c r="H78">
-        <v>4.583333333333336</v>
+        <v>1</v>
       </c>
       <c r="I78">
         <v>2023</v>
@@ -4502,7 +4466,7 @@
         <v>2015</v>
       </c>
       <c r="O78">
-        <v>92.82666666666668</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="79">
@@ -4573,7 +4537,7 @@
         </is>
       </c>
       <c r="H80">
-        <v>-0.7051282051282612</v>
+        <v>-0.6749999999999972</v>
       </c>
       <c r="I80">
         <v>2023</v>
@@ -4598,7 +4562,7 @@
         <v>2015</v>
       </c>
       <c r="O80">
-        <v>67</v>
+        <v>67.80000000000022</v>
       </c>
     </row>
     <row r="81">
@@ -4627,7 +4591,7 @@
         </is>
       </c>
       <c r="H81">
-        <v>0.6352758831207055</v>
+        <v>0.4687499999999929</v>
       </c>
       <c r="I81">
         <v>2023</v>
@@ -4652,7 +4616,7 @@
         <v>2015</v>
       </c>
       <c r="O81">
-        <v>80.14483284914326</v>
+        <v>80.67500000000008</v>
       </c>
     </row>
     <row r="82">
@@ -4681,7 +4645,7 @@
         </is>
       </c>
       <c r="H82">
-        <v>-1.15384352237799</v>
+        <v>-0.8645833333333215</v>
       </c>
       <c r="I82">
         <v>2023</v>
@@ -4706,7 +4670,7 @@
         <v>2015</v>
       </c>
       <c r="O82">
-        <v>81.52250836120407</v>
+        <v>82.00000000000014</v>
       </c>
     </row>
     <row r="83">
@@ -4735,7 +4699,7 @@
         </is>
       </c>
       <c r="H83">
-        <v>0.861724519353217</v>
+        <v>0.71875</v>
       </c>
       <c r="I83">
         <v>2023</v>
@@ -4760,7 +4724,7 @@
         <v>2015</v>
       </c>
       <c r="O83">
-        <v>76.54604819200404</v>
+        <v>77.10000000000001</v>
       </c>
     </row>
     <row r="84">
@@ -4789,7 +4753,7 @@
         </is>
       </c>
       <c r="H84">
-        <v>-2.533042452401162</v>
+        <v>-1.999999999999979</v>
       </c>
       <c r="I84">
         <v>2023</v>
@@ -4814,7 +4778,7 @@
         <v>2015</v>
       </c>
       <c r="O84">
-        <v>81.86773913043484</v>
+        <v>82.40000000000015</v>
       </c>
     </row>
     <row r="85">
@@ -4843,7 +4807,7 @@
         </is>
       </c>
       <c r="H85">
-        <v>-2.517018785401149</v>
+        <v>-2.1875</v>
       </c>
       <c r="I85">
         <v>2023</v>
@@ -4868,7 +4832,7 @@
         <v>2015</v>
       </c>
       <c r="O85">
-        <v>61.73479374110966</v>
+        <v>61.90000000000001</v>
       </c>
     </row>
     <row r="86">
@@ -4897,7 +4861,7 @@
         </is>
       </c>
       <c r="H86">
-        <v>1.254370629370626</v>
+        <v>0.75</v>
       </c>
       <c r="I86">
         <v>2023</v>
@@ -4922,7 +4886,7 @@
         <v>2015</v>
       </c>
       <c r="O86">
-        <v>87.17615384615387</v>
+        <v>87.80000000000001</v>
       </c>
     </row>
     <row r="87">
@@ -4951,7 +4915,7 @@
         </is>
       </c>
       <c r="H87">
-        <v>-0.4464285714285765</v>
+        <v>-0.4166666666666785</v>
       </c>
       <c r="I87">
         <v>2023</v>
@@ -4976,7 +4940,7 @@
         <v>2015</v>
       </c>
       <c r="O87">
-        <v>43.41999999999989</v>
+        <v>43.49999999999993</v>
       </c>
     </row>
     <row r="88">
@@ -5005,7 +4969,7 @@
         </is>
       </c>
       <c r="H88">
-        <v>1.134492607526845</v>
+        <v>1.1666666666667</v>
       </c>
       <c r="I88">
         <v>2023</v>
@@ -5030,7 +4994,7 @@
         <v>2015</v>
       </c>
       <c r="O88">
-        <v>49.26333333333343</v>
+        <v>49.19999999999993</v>
       </c>
     </row>
     <row r="89">
@@ -5059,7 +5023,7 @@
         </is>
       </c>
       <c r="H89">
-        <v>1.903479137031681</v>
+        <v>1.75</v>
       </c>
       <c r="I89">
         <v>2023</v>
@@ -5084,7 +5048,7 @@
         <v>2015</v>
       </c>
       <c r="O89">
-        <v>58.47833333333339</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="90">
@@ -5113,7 +5077,7 @@
         </is>
       </c>
       <c r="H90">
-        <v>-1.010728414172682</v>
+        <v>-0.6249999999999645</v>
       </c>
       <c r="I90">
         <v>2023</v>
@@ -5138,7 +5102,7 @@
         <v>2015</v>
       </c>
       <c r="O90">
-        <v>85.37279411764706</v>
+        <v>85.73333333333335</v>
       </c>
     </row>
     <row r="91">
@@ -5167,7 +5131,7 @@
         </is>
       </c>
       <c r="H91">
-        <v>1.525862068965523</v>
+        <v>1.500000000000043</v>
       </c>
       <c r="I91">
         <v>2023</v>
@@ -5192,7 +5156,7 @@
         <v>2015</v>
       </c>
       <c r="O91">
-        <v>45.13793103448266</v>
+        <v>45.19999999999993</v>
       </c>
     </row>
     <row r="92">
@@ -5221,7 +5185,7 @@
         </is>
       </c>
       <c r="H92">
-        <v>-1.940061139074309</v>
+        <v>-1.587499999999935</v>
       </c>
       <c r="I92">
         <v>2023</v>
@@ -5246,7 +5210,7 @@
         <v>2015</v>
       </c>
       <c r="O92">
-        <v>74.91748605748607</v>
+        <v>75.3</v>
       </c>
     </row>
     <row r="93">
@@ -5275,7 +5239,7 @@
         </is>
       </c>
       <c r="H93">
-        <v>0.6800536420101437</v>
+        <v>0.4999999999999716</v>
       </c>
       <c r="I93">
         <v>2023</v>
@@ -5300,7 +5264,7 @@
         <v>2015</v>
       </c>
       <c r="O93">
-        <v>82.72143798230759</v>
+        <v>83.40000000000015</v>
       </c>
     </row>
     <row r="94">
@@ -5329,7 +5293,7 @@
         </is>
       </c>
       <c r="H94">
-        <v>9.562499999999993</v>
+        <v>3.25</v>
       </c>
       <c r="I94">
         <v>2023</v>
@@ -5354,7 +5318,7 @@
         <v>2015</v>
       </c>
       <c r="O94">
-        <v>91.01666666666667</v>
+        <v>91.40000000000001</v>
       </c>
     </row>
     <row r="95">
@@ -5383,7 +5347,7 @@
         </is>
       </c>
       <c r="H95">
-        <v>4.743055555555571</v>
+        <v>3</v>
       </c>
       <c r="I95">
         <v>2023</v>
@@ -5408,7 +5372,7 @@
         <v>2015</v>
       </c>
       <c r="O95">
-        <v>89.08444444444446</v>
+        <v>89.40000000000001</v>
       </c>
     </row>
     <row r="96">
@@ -5479,7 +5443,7 @@
         </is>
       </c>
       <c r="H97">
-        <v>1.721152422777784</v>
+        <v>1.524999999999999</v>
       </c>
       <c r="I97">
         <v>2023</v>
@@ -5504,7 +5468,7 @@
         <v>2015</v>
       </c>
       <c r="O97">
-        <v>73.53460565829002</v>
+        <v>73.81999999999998</v>
       </c>
     </row>
     <row r="98">
@@ -5533,7 +5497,7 @@
         </is>
       </c>
       <c r="H98">
-        <v>7.952651515151537</v>
+        <v>4.625</v>
       </c>
       <c r="I98">
         <v>2023</v>
@@ -5558,7 +5522,7 @@
         <v>2015</v>
       </c>
       <c r="O98">
-        <v>87.70454545454545</v>
+        <v>88.40000000000001</v>
       </c>
     </row>
     <row r="99">
@@ -5587,7 +5551,7 @@
         </is>
       </c>
       <c r="H99">
-        <v>-3.062117956476655</v>
+        <v>-2.47916666666665</v>
       </c>
       <c r="I99">
         <v>2023</v>
@@ -5612,7 +5576,7 @@
         <v>2015</v>
       </c>
       <c r="O99">
-        <v>81.69173913043481</v>
+        <v>82.20000000000014</v>
       </c>
     </row>
     <row r="100">
@@ -5641,7 +5605,7 @@
         </is>
       </c>
       <c r="H100">
-        <v>3.267174031855717</v>
+        <v>2.84375</v>
       </c>
       <c r="I100">
         <v>2023</v>
@@ -5666,7 +5630,7 @@
         <v>2015</v>
       </c>
       <c r="O100">
-        <v>53.42473484848477</v>
+        <v>54</v>
       </c>
     </row>
     <row r="101">
@@ -5695,7 +5659,7 @@
         </is>
       </c>
       <c r="H101">
-        <v>1.069896611314149</v>
+        <v>0.8125</v>
       </c>
       <c r="I101">
         <v>2023</v>
@@ -5720,7 +5684,7 @@
         <v>2015</v>
       </c>
       <c r="O101">
-        <v>78.14141129032259</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="102">
@@ -5749,7 +5713,7 @@
         </is>
       </c>
       <c r="H102">
-        <v>-1.364174836601293</v>
+        <v>-0.9791666666666501</v>
       </c>
       <c r="I102">
         <v>2023</v>
@@ -5774,7 +5738,7 @@
         <v>2015</v>
       </c>
       <c r="O102">
-        <v>86.40238095238095</v>
+        <v>86.90000000000001</v>
       </c>
     </row>
     <row r="103">
@@ -5803,7 +5767,7 @@
         </is>
       </c>
       <c r="H103">
-        <v>0.3956258890469115</v>
+        <v>0.3374999999999915</v>
       </c>
       <c r="I103">
         <v>2023</v>
@@ -5828,7 +5792,7 @@
         <v>2015</v>
       </c>
       <c r="O103">
-        <v>73.06762446657198</v>
+        <v>73.42000000000007</v>
       </c>
     </row>
     <row r="104">
@@ -5857,7 +5821,7 @@
         </is>
       </c>
       <c r="H104">
-        <v>9.985854219310127</v>
+        <v>6.166666666666664</v>
       </c>
       <c r="I104">
         <v>2023</v>
@@ -5882,7 +5846,7 @@
         <v>2015</v>
       </c>
       <c r="O104">
-        <v>85.37279411764706</v>
+        <v>85.73333333333335</v>
       </c>
     </row>
     <row r="105">
@@ -5911,7 +5875,7 @@
         </is>
       </c>
       <c r="H105">
-        <v>-9.829553634817312</v>
+        <v>-9.145833333333524</v>
       </c>
       <c r="I105">
         <v>2023</v>
@@ -5936,7 +5900,7 @@
         <v>2015</v>
       </c>
       <c r="O105">
-        <v>61.00216216216231</v>
+        <v>61.2</v>
       </c>
     </row>
     <row r="106">
@@ -5965,7 +5929,7 @@
         </is>
       </c>
       <c r="H106">
-        <v>0.8795426065163028</v>
+        <v>0.5833333333333002</v>
       </c>
       <c r="I106">
         <v>2023</v>
@@ -5990,7 +5954,7 @@
         <v>2015</v>
       </c>
       <c r="O106">
-        <v>83.57345864661653</v>
+        <v>84.3333333333334</v>
       </c>
     </row>
     <row r="107">
@@ -6019,7 +5983,7 @@
         </is>
       </c>
       <c r="H107">
-        <v>-6.133886754482518</v>
+        <v>-4.312499999999879</v>
       </c>
       <c r="I107">
         <v>2023</v>
@@ -6044,7 +6008,7 @@
         <v>2015</v>
       </c>
       <c r="O107">
-        <v>88.13636363636363</v>
+        <v>88.85000000000001</v>
       </c>
     </row>
     <row r="108">
@@ -6073,7 +6037,7 @@
         </is>
       </c>
       <c r="H108">
-        <v>-0.1439075630252091</v>
+        <v>-0.125</v>
       </c>
       <c r="I108">
         <v>2023</v>
@@ -6098,7 +6062,7 @@
         <v>2015</v>
       </c>
       <c r="O108">
-        <v>76.90293894830657</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="109">
@@ -6127,7 +6091,7 @@
         </is>
       </c>
       <c r="H109">
-        <v>0.625</v>
+        <v>0.4999999999999716</v>
       </c>
       <c r="I109">
         <v>2023</v>
@@ -6152,7 +6116,7 @@
         <v>2015</v>
       </c>
       <c r="O109">
-        <v>67.49750000000003</v>
+        <v>68.30000000000022</v>
       </c>
     </row>
     <row r="110">
@@ -6181,7 +6145,7 @@
         </is>
       </c>
       <c r="H110">
-        <v>-2.536636110848967</v>
+        <v>-1.916666666666579</v>
       </c>
       <c r="I110">
         <v>2023</v>
@@ -6206,7 +6170,7 @@
         <v>2015</v>
       </c>
       <c r="O110">
-        <v>84.25540935672517</v>
+        <v>84.8666666666667</v>
       </c>
     </row>
     <row r="111">
@@ -6235,7 +6199,7 @@
         </is>
       </c>
       <c r="H111">
-        <v>0.2543103448275872</v>
+        <v>0.1875</v>
       </c>
       <c r="I111">
         <v>2023</v>
@@ -6260,7 +6224,7 @@
         <v>2015</v>
       </c>
       <c r="O111">
-        <v>79.54000547345375</v>
+        <v>80.15000000000008</v>
       </c>
     </row>
     <row r="112">
@@ -6289,7 +6253,7 @@
         </is>
       </c>
       <c r="H112">
-        <v>4.732859294981175</v>
+        <v>3.837499999999928</v>
       </c>
       <c r="I112">
         <v>2023</v>
@@ -6314,7 +6278,7 @@
         <v>2015</v>
       </c>
       <c r="O112">
-        <v>68.7649999999999</v>
+        <v>69.60000000000024</v>
       </c>
     </row>
     <row r="113">
@@ -6343,7 +6307,7 @@
         </is>
       </c>
       <c r="H113">
-        <v>-0.2777777777777715</v>
+        <v>-0.1666666666666572</v>
       </c>
       <c r="I113">
         <v>2023</v>
@@ -6368,7 +6332,7 @@
         <v>2015</v>
       </c>
       <c r="O113">
-        <v>85.11299019607844</v>
+        <v>85.53333333333335</v>
       </c>
     </row>
     <row r="114">
@@ -6397,7 +6361,7 @@
         </is>
       </c>
       <c r="H114">
-        <v>-2.000421657155371</v>
+        <v>-1.718749999999972</v>
       </c>
       <c r="I114">
         <v>2023</v>
@@ -6422,7 +6386,7 @@
         <v>2015</v>
       </c>
       <c r="O114">
-        <v>77.17077583232705</v>
+        <v>77.80000000000001</v>
       </c>
     </row>
     <row r="115">
@@ -6451,7 +6415,7 @@
         </is>
       </c>
       <c r="H115">
-        <v>-0.5762999841946979</v>
+        <v>-0.53125</v>
       </c>
       <c r="I115">
         <v>2023</v>
@@ -6476,7 +6440,7 @@
         <v>2015</v>
       </c>
       <c r="O115">
-        <v>75.46495798319326</v>
+        <v>75.90000000000001</v>
       </c>
     </row>
     <row r="116">
@@ -6505,7 +6469,7 @@
         </is>
       </c>
       <c r="H116">
-        <v>-5.931243906771059</v>
+        <v>-5.118749999999899</v>
       </c>
       <c r="I116">
         <v>2023</v>
@@ -6530,7 +6494,7 @@
         <v>2015</v>
       </c>
       <c r="O116">
-        <v>78.84375258223426</v>
+        <v>79.55000000000004</v>
       </c>
     </row>
     <row r="117">
@@ -6559,7 +6523,7 @@
         </is>
       </c>
       <c r="H117">
-        <v>-2.166666666666671</v>
+        <v>-1.125</v>
       </c>
       <c r="I117">
         <v>2023</v>
@@ -6584,7 +6548,7 @@
         <v>2015</v>
       </c>
       <c r="O117">
-        <v>91.72</v>
+        <v>92.2</v>
       </c>
     </row>
     <row r="118">
@@ -6655,7 +6619,7 @@
         </is>
       </c>
       <c r="H119">
-        <v>-0.5532635467980285</v>
+        <v>-0.40625</v>
       </c>
       <c r="I119">
         <v>2023</v>
@@ -6680,7 +6644,7 @@
         <v>2015</v>
       </c>
       <c r="O119">
-        <v>80.40227106227114</v>
+        <v>80.90000000000015</v>
       </c>
     </row>
     <row r="120">
@@ -6751,7 +6715,7 @@
         </is>
       </c>
       <c r="H121">
-        <v>-0.1785714285714306</v>
+        <v>-0.1666666666666714</v>
       </c>
       <c r="I121">
         <v>2023</v>
@@ -6776,7 +6740,7 @@
         <v>2015</v>
       </c>
       <c r="O121">
-        <v>39.73999999999999</v>
+        <v>39.89999999999993</v>
       </c>
     </row>
     <row r="122">
@@ -6805,7 +6769,7 @@
         </is>
       </c>
       <c r="H122">
-        <v>-1.388493756914748</v>
+        <v>-1.28125</v>
       </c>
       <c r="I122">
         <v>2023</v>
@@ -6830,7 +6794,7 @@
         <v>2015</v>
       </c>
       <c r="O122">
-        <v>63.60157894736831</v>
+        <v>63.72499999999997</v>
       </c>
     </row>
     <row r="123">
@@ -6859,7 +6823,7 @@
         </is>
       </c>
       <c r="H123">
-        <v>-1.651610271757619</v>
+        <v>-1.270833333333307</v>
       </c>
       <c r="I123">
         <v>2023</v>
@@ -6884,7 +6848,7 @@
         <v>2015</v>
       </c>
       <c r="O123">
-        <v>82.03720553359686</v>
+        <v>82.60000000000015</v>
       </c>
     </row>
     <row r="124">
@@ -6913,7 +6877,7 @@
         </is>
       </c>
       <c r="H124">
-        <v>1.650578328052063</v>
+        <v>1.291666666666615</v>
       </c>
       <c r="I124">
         <v>2023</v>
@@ -6938,7 +6902,7 @@
         <v>2015</v>
       </c>
       <c r="O124">
-        <v>80.05862595259154</v>
+        <v>80.60000000000008</v>
       </c>
     </row>
     <row r="125">
@@ -6967,7 +6931,7 @@
         </is>
       </c>
       <c r="H125">
-        <v>-2.600390736611516</v>
+        <v>-1.812499999999915</v>
       </c>
       <c r="I125">
         <v>2023</v>
@@ -6992,7 +6956,7 @@
         <v>2015</v>
       </c>
       <c r="O125">
-        <v>85.89083333333332</v>
+        <v>86.30000000000001</v>
       </c>
     </row>
     <row r="126">
@@ -7021,7 +6985,7 @@
         </is>
       </c>
       <c r="H126">
-        <v>0.6048387096774022</v>
+        <v>0.6250000000000178</v>
       </c>
       <c r="I126">
         <v>2023</v>
@@ -7046,7 +7010,7 @@
         <v>2015</v>
       </c>
       <c r="O126">
-        <v>49.78903225806455</v>
+        <v>49.69999999999993</v>
       </c>
     </row>
     <row r="127">
@@ -7075,7 +7039,7 @@
         </is>
       </c>
       <c r="H127">
-        <v>-17.359015984016</v>
+        <v>-7.875</v>
       </c>
       <c r="I127">
         <v>2023</v>
@@ -7100,7 +7064,7 @@
         <v>2015</v>
       </c>
       <c r="O127">
-        <v>93.46000000000001</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="128">
@@ -7129,7 +7093,7 @@
         </is>
       </c>
       <c r="H128">
-        <v>1.002083333333346</v>
+        <v>0.833333333333357</v>
       </c>
       <c r="I128">
         <v>2023</v>
@@ -7154,7 +7118,7 @@
         <v>2015</v>
       </c>
       <c r="O128">
-        <v>29.89583333333328</v>
+        <v>30.29999999999993</v>
       </c>
     </row>
     <row r="129">
@@ -7183,7 +7147,7 @@
         </is>
       </c>
       <c r="H129">
-        <v>-11.54166666666669</v>
+        <v>-4.875</v>
       </c>
       <c r="I129">
         <v>2023</v>
@@ -7208,7 +7172,7 @@
         <v>2015</v>
       </c>
       <c r="O129">
-        <v>93.26000000000001</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="130">
@@ -7237,7 +7201,7 @@
         </is>
       </c>
       <c r="H130">
-        <v>0.3645092460881685</v>
+        <v>0.3249999999999957</v>
       </c>
       <c r="I130">
         <v>2023</v>
@@ -7262,7 +7226,7 @@
         <v>2015</v>
       </c>
       <c r="O130">
-        <v>73.3503951319742</v>
+        <v>73.66000000000004</v>
       </c>
     </row>
     <row r="131">
@@ -7291,7 +7255,7 @@
         </is>
       </c>
       <c r="H131">
-        <v>-1.611651835372562</v>
+        <v>-1.625000000000046</v>
       </c>
       <c r="I131">
         <v>2023</v>
@@ -7316,7 +7280,7 @@
         <v>2015</v>
       </c>
       <c r="O131">
-        <v>50.92451612903228</v>
+        <v>50.99999999999991</v>
       </c>
     </row>
     <row r="132">
@@ -7345,7 +7309,7 @@
         </is>
       </c>
       <c r="H132">
-        <v>-1.542628205128221</v>
+        <v>-1.291666666666703</v>
       </c>
       <c r="I132">
         <v>2023</v>
@@ -7370,7 +7334,7 @@
         <v>2015</v>
       </c>
       <c r="O132">
-        <v>32.98</v>
+        <v>33.29999999999993</v>
       </c>
     </row>
     <row r="133">
@@ -7399,7 +7363,7 @@
         </is>
       </c>
       <c r="H133">
-        <v>2.046989468864474</v>
+        <v>1.375</v>
       </c>
       <c r="I133">
         <v>2023</v>
@@ -7424,7 +7388,7 @@
         <v>2015</v>
       </c>
       <c r="O133">
-        <v>86.06113095238094</v>
+        <v>86.5</v>
       </c>
     </row>
     <row r="134">
@@ -7453,7 +7417,7 @@
         </is>
       </c>
       <c r="H134">
-        <v>-4.060530419083072</v>
+        <v>-3.581249999999926</v>
       </c>
       <c r="I134">
         <v>2023</v>
@@ -7478,7 +7442,7 @@
         <v>2015</v>
       </c>
       <c r="O134">
-        <v>71.84812415654528</v>
+        <v>72.38000000000011</v>
       </c>
     </row>
     <row r="135">
@@ -7507,7 +7471,7 @@
         </is>
       </c>
       <c r="H135">
-        <v>-8.25740787230437</v>
+        <v>-6.6187499999998</v>
       </c>
       <c r="I135">
         <v>2023</v>
@@ -7532,7 +7496,7 @@
         <v>2015</v>
       </c>
       <c r="O135">
-        <v>84.68075679394569</v>
+        <v>85.20000000000005</v>
       </c>
     </row>
     <row r="136">
@@ -7561,7 +7525,7 @@
         </is>
       </c>
       <c r="H136">
-        <v>4.472010869565224</v>
+        <v>4.354166666666732</v>
       </c>
       <c r="I136">
         <v>2023</v>
@@ -7586,7 +7550,7 @@
         <v>2015</v>
       </c>
       <c r="O136">
-        <v>25.94173913043477</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="137">
@@ -7615,7 +7579,7 @@
         </is>
       </c>
       <c r="H137">
-        <v>-6.093210724460807</v>
+        <v>-5.395833333333485</v>
       </c>
       <c r="I137">
         <v>2023</v>
@@ -7640,7 +7604,7 @@
         <v>2015</v>
       </c>
       <c r="O137">
-        <v>42.48785714285707</v>
+        <v>42.59999999999993</v>
       </c>
     </row>
     <row r="138">
@@ -7669,7 +7633,7 @@
         </is>
       </c>
       <c r="H138">
-        <v>2.169577767004235</v>
+        <v>1.54166666666665</v>
       </c>
       <c r="I138">
         <v>2023</v>
@@ -7694,7 +7658,7 @@
         <v>2015</v>
       </c>
       <c r="O138">
-        <v>84.85385620915036</v>
+        <v>85.33333333333336</v>
       </c>
     </row>
     <row r="139">
@@ -7723,7 +7687,7 @@
         </is>
       </c>
       <c r="H139">
-        <v>-1.15506715506713</v>
+        <v>-0.9166666666666288</v>
       </c>
       <c r="I139">
         <v>2023</v>
@@ -7748,7 +7712,7 @@
         <v>2015</v>
       </c>
       <c r="O139">
-        <v>82.46781479390179</v>
+        <v>83.10000000000015</v>
       </c>
     </row>
     <row r="140">
@@ -7777,7 +7741,7 @@
         </is>
       </c>
       <c r="H140">
-        <v>7.720462011433369</v>
+        <v>7.137500000000045</v>
       </c>
       <c r="I140">
         <v>2023</v>
@@ -7802,7 +7766,7 @@
         <v>2015</v>
       </c>
       <c r="O140">
-        <v>46.58620689655181</v>
+        <v>46.59999999999993</v>
       </c>
     </row>
     <row r="141">
@@ -7831,7 +7795,7 @@
         </is>
       </c>
       <c r="H141">
-        <v>1.543148276843894</v>
+        <v>1.218749999999943</v>
       </c>
       <c r="I141">
         <v>2023</v>
@@ -7856,7 +7820,7 @@
         <v>2015</v>
       </c>
       <c r="O141">
-        <v>80.48798534798541</v>
+        <v>80.97500000000011</v>
       </c>
     </row>
     <row r="142">
@@ -7885,7 +7849,7 @@
         </is>
       </c>
       <c r="H142">
-        <v>-8.147870247804384</v>
+        <v>-7.024999999999899</v>
       </c>
       <c r="I142">
         <v>2023</v>
@@ -7910,7 +7874,7 @@
         <v>2015</v>
       </c>
       <c r="O142">
-        <v>79.80000526293634</v>
+        <v>80.37500000000009</v>
       </c>
     </row>
     <row r="143">
@@ -7939,7 +7903,7 @@
         </is>
       </c>
       <c r="H143">
-        <v>6.242020248270318</v>
+        <v>5.645833333333478</v>
       </c>
       <c r="I143">
         <v>2023</v>
@@ -7964,7 +7928,7 @@
         <v>2015</v>
       </c>
       <c r="O143">
-        <v>28.43750000000001</v>
+        <v>28.44999999999997</v>
       </c>
     </row>
     <row r="144">
@@ -7993,7 +7957,7 @@
         </is>
       </c>
       <c r="H144">
-        <v>4.126377095127104</v>
+        <v>2.4375</v>
       </c>
       <c r="I144">
         <v>2023</v>
@@ -8018,7 +7982,7 @@
         <v>2015</v>
       </c>
       <c r="O144">
-        <v>85.97833333333332</v>
+        <v>86.40000000000001</v>
       </c>
     </row>
     <row r="145">
@@ -8047,7 +8011,7 @@
         </is>
       </c>
       <c r="H145">
-        <v>-1.331588669950747</v>
+        <v>-1.250000000000036</v>
       </c>
       <c r="I145">
         <v>2023</v>
@@ -8072,7 +8036,7 @@
         <v>2015</v>
       </c>
       <c r="O145">
-        <v>43.91999999999987</v>
+        <v>43.99999999999993</v>
       </c>
     </row>
     <row r="146">
@@ -8101,7 +8065,7 @@
         </is>
       </c>
       <c r="H146">
-        <v>3.010131584531742</v>
+        <v>2.104166666666607</v>
       </c>
       <c r="I146">
         <v>2023</v>
@@ -8126,7 +8090,7 @@
         <v>2015</v>
       </c>
       <c r="O146">
-        <v>83.31989177489177</v>
+        <v>84.10000000000015</v>
       </c>
     </row>
     <row r="147">
@@ -8155,7 +8119,7 @@
         </is>
       </c>
       <c r="H147">
-        <v>2.839983749910211</v>
+        <v>1.958333333333314</v>
       </c>
       <c r="I147">
         <v>2023</v>
@@ -8180,7 +8144,7 @@
         <v>2015</v>
       </c>
       <c r="O147">
-        <v>84.76496732026146</v>
+        <v>85.26666666666671</v>
       </c>
     </row>
     <row r="148">
@@ -8209,7 +8173,7 @@
         </is>
       </c>
       <c r="H148">
-        <v>2.788690476190467</v>
+        <v>1.8125</v>
       </c>
       <c r="I148">
         <v>2023</v>
@@ -8234,7 +8198,7 @@
         <v>2015</v>
       </c>
       <c r="O148">
-        <v>88.82666666666668</v>
+        <v>89.25</v>
       </c>
     </row>
     <row r="149">
@@ -8262,17 +8226,11 @@
           <t>SVN</t>
         </is>
       </c>
-      <c r="H149">
-        <v>-6.25</v>
-      </c>
       <c r="I149">
         <v>2023</v>
       </c>
       <c r="J149">
-        <v>93.80000000000001</v>
-      </c>
-      <c r="K149">
-        <v>94.30000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -8283,9 +8241,6 @@
         <is>
           <t>Women political empowerment index</t>
         </is>
-      </c>
-      <c r="N149">
-        <v>2015</v>
       </c>
     </row>
     <row r="150">
@@ -8356,7 +8311,7 @@
         </is>
       </c>
       <c r="H151">
-        <v>-1.714743589743609</v>
+        <v>-1.500000000000043</v>
       </c>
       <c r="I151">
         <v>2023</v>
@@ -8381,7 +8336,7 @@
         <v>2015</v>
       </c>
       <c r="O151">
-        <v>36.15999999999995</v>
+        <v>36.39999999999993</v>
       </c>
     </row>
     <row r="152">
@@ -8410,7 +8365,7 @@
         </is>
       </c>
       <c r="H152">
-        <v>4.630681818181834</v>
+        <v>2.875</v>
       </c>
       <c r="I152">
         <v>2023</v>
@@ -8435,7 +8390,7 @@
         <v>2015</v>
       </c>
       <c r="O152">
-        <v>88.04545454545453</v>
+        <v>88.80000000000001</v>
       </c>
     </row>
     <row r="153">
@@ -8464,7 +8419,7 @@
         </is>
       </c>
       <c r="H153">
-        <v>-0.961538461538467</v>
+        <v>-0.833333333333357</v>
       </c>
       <c r="I153">
         <v>2023</v>
@@ -8489,7 +8444,7 @@
         <v>2015</v>
       </c>
       <c r="O153">
-        <v>34.9484615384615</v>
+        <v>35.19999999999993</v>
       </c>
     </row>
     <row r="154">
@@ -8518,7 +8473,7 @@
         </is>
       </c>
       <c r="H154">
-        <v>1.871855961445689</v>
+        <v>1.6875</v>
       </c>
       <c r="I154">
         <v>2023</v>
@@ -8543,7 +8498,7 @@
         <v>2015</v>
       </c>
       <c r="O154">
-        <v>57.31949579831938</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="155">
@@ -8572,7 +8527,7 @@
         </is>
       </c>
       <c r="H155">
-        <v>-3.236234380593075</v>
+        <v>-2.645833333333321</v>
       </c>
       <c r="I155">
         <v>2023</v>
@@ -8597,7 +8552,7 @@
         <v>2015</v>
       </c>
       <c r="O155">
-        <v>81.52250836120407</v>
+        <v>82.00000000000014</v>
       </c>
     </row>
     <row r="156">
@@ -8626,7 +8581,7 @@
         </is>
       </c>
       <c r="H156">
-        <v>0.4166666666666998</v>
+        <v>0.3249999999999815</v>
       </c>
       <c r="I156">
         <v>2023</v>
@@ -8651,7 +8606,7 @@
         <v>2015</v>
       </c>
       <c r="O156">
-        <v>70.50153846153836</v>
+        <v>71.26000000000013</v>
       </c>
     </row>
     <row r="157">
@@ -8680,7 +8635,7 @@
         </is>
       </c>
       <c r="H157">
-        <v>-2.056590656284733</v>
+        <v>-2.041666666666725</v>
       </c>
       <c r="I157">
         <v>2023</v>
@@ -8705,7 +8660,7 @@
         <v>2015</v>
       </c>
       <c r="O157">
-        <v>50.40838709677425</v>
+        <v>50.33333333333321</v>
       </c>
     </row>
     <row r="158">
@@ -8734,7 +8689,7 @@
         </is>
       </c>
       <c r="H158">
-        <v>2.255233990147822</v>
+        <v>2.12500000000006</v>
       </c>
       <c r="I158">
         <v>2023</v>
@@ -8759,7 +8714,7 @@
         <v>2015</v>
       </c>
       <c r="O158">
-        <v>39.63999999999999</v>
+        <v>39.79999999999993</v>
       </c>
     </row>
     <row r="159">
@@ -8788,7 +8743,7 @@
         </is>
       </c>
       <c r="H159">
-        <v>1.554966266135338</v>
+        <v>1.25</v>
       </c>
       <c r="I159">
         <v>2023</v>
@@ -8813,7 +8768,7 @@
         <v>2015</v>
       </c>
       <c r="O159">
-        <v>76.45747676343261</v>
+        <v>77</v>
       </c>
     </row>
     <row r="160">
@@ -8842,7 +8797,7 @@
         </is>
       </c>
       <c r="H160">
-        <v>-4.138777888777881</v>
+        <v>-2.4375</v>
       </c>
       <c r="I160">
         <v>2023</v>
@@ -8867,7 +8822,7 @@
         <v>2015</v>
       </c>
       <c r="O160">
-        <v>89.78500000000001</v>
+        <v>90</v>
       </c>
     </row>
     <row r="161">
@@ -8896,7 +8851,7 @@
         </is>
       </c>
       <c r="H161">
-        <v>-4.244778522600647</v>
+        <v>-3.104166666666551</v>
       </c>
       <c r="I161">
         <v>2023</v>
@@ -8921,7 +8876,7 @@
         <v>2015</v>
       </c>
       <c r="O161">
-        <v>85.28455882352944</v>
+        <v>85.6666666666667</v>
       </c>
     </row>
     <row r="162">
@@ -8950,7 +8905,7 @@
         </is>
       </c>
       <c r="H162">
-        <v>-1.771938942991561</v>
+        <v>-1.6875</v>
       </c>
       <c r="I162">
         <v>2023</v>
@@ -8975,7 +8930,7 @@
         <v>2015</v>
       </c>
       <c r="O162">
-        <v>66.48717948717949</v>
+        <v>67.22500000000019</v>
       </c>
     </row>
     <row r="163">
@@ -9004,7 +8959,7 @@
         </is>
       </c>
       <c r="H163">
-        <v>1.250000000000014</v>
+        <v>0.75</v>
       </c>
       <c r="I163">
         <v>2023</v>
@@ -9029,7 +8984,7 @@
         <v>2015</v>
       </c>
       <c r="O163">
-        <v>90.58</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="164">
@@ -9058,7 +9013,7 @@
         </is>
       </c>
       <c r="H164">
-        <v>2.444140736611509</v>
+        <v>1.687499999999922</v>
       </c>
       <c r="I164">
         <v>2023</v>
@@ -9083,7 +9038,7 @@
         <v>2015</v>
       </c>
       <c r="O164">
-        <v>82.63448146056845</v>
+        <v>83.30000000000015</v>
       </c>
     </row>
     <row r="165">
@@ -9112,7 +9067,7 @@
         </is>
       </c>
       <c r="H165">
-        <v>-3.426059932147318</v>
+        <v>-2.849999999999959</v>
       </c>
       <c r="I165">
         <v>2023</v>
@@ -9137,7 +9092,7 @@
         <v>2015</v>
       </c>
       <c r="O165">
-        <v>79.71333880678711</v>
+        <v>80.30000000000008</v>
       </c>
     </row>
     <row r="166">
@@ -9166,7 +9121,7 @@
         </is>
       </c>
       <c r="H166">
-        <v>6.172177871578022</v>
+        <v>3.791666666666615</v>
       </c>
       <c r="I166">
         <v>2023</v>
@@ -9191,7 +9146,7 @@
         <v>2015</v>
       </c>
       <c r="O166">
-        <v>83.57345864661653</v>
+        <v>84.3333333333334</v>
       </c>
     </row>
     <row r="167">
@@ -9220,7 +9175,7 @@
         </is>
       </c>
       <c r="H167">
-        <v>-3.159722222222243</v>
+        <v>-2.1875</v>
       </c>
       <c r="I167">
         <v>2023</v>
@@ -9245,7 +9200,7 @@
         <v>2015</v>
       </c>
       <c r="O167">
-        <v>90.93333333333332</v>
+        <v>91.30000000000001</v>
       </c>
     </row>
     <row r="168">
@@ -9274,7 +9229,7 @@
         </is>
       </c>
       <c r="H168">
-        <v>-0.892857142857153</v>
+        <v>-0.625</v>
       </c>
       <c r="I168">
         <v>2023</v>
@@ -9299,7 +9254,7 @@
         <v>2015</v>
       </c>
       <c r="O168">
-        <v>90.40857142857143</v>
+        <v>90.7</v>
       </c>
     </row>
     <row r="169">
@@ -9328,7 +9283,7 @@
         </is>
       </c>
       <c r="H169">
-        <v>5.418763944136451</v>
+        <v>4.804166666666646</v>
       </c>
       <c r="I169">
         <v>2023</v>
@@ -9353,7 +9308,7 @@
         <v>2015</v>
       </c>
       <c r="O169">
-        <v>52.386875</v>
+        <v>52.86666666666661</v>
       </c>
     </row>
     <row r="170">
@@ -9382,7 +9337,7 @@
         </is>
       </c>
       <c r="H170">
-        <v>-0.224867724867714</v>
+        <v>-0.15625</v>
       </c>
       <c r="I170">
         <v>2023</v>
@@ -9407,7 +9362,7 @@
         <v>2015</v>
       </c>
       <c r="O170">
-        <v>80.83401709401714</v>
+        <v>81.27500000000011</v>
       </c>
     </row>
     <row r="171">
@@ -9436,7 +9391,7 @@
         </is>
       </c>
       <c r="H171">
-        <v>0.1470588235294201</v>
+        <v>0.125</v>
       </c>
       <c r="I171">
         <v>2023</v>
@@ -9461,7 +9416,7 @@
         <v>2015</v>
       </c>
       <c r="O171">
-        <v>76.99411541889479</v>
+        <v>77.60000000000001</v>
       </c>
     </row>
     <row r="172">
@@ -9490,7 +9445,7 @@
         </is>
       </c>
       <c r="H172">
-        <v>1.017628205128261</v>
+        <v>0.7999999999999545</v>
       </c>
       <c r="I172">
         <v>2023</v>
@@ -9515,7 +9470,7 @@
         <v>2015</v>
       </c>
       <c r="O172">
-        <v>69.54499999999986</v>
+        <v>70.40000000000023</v>
       </c>
     </row>
     <row r="173">
@@ -9544,7 +9499,7 @@
         </is>
       </c>
       <c r="H173">
-        <v>1.880777954989284</v>
+        <v>1.625</v>
       </c>
       <c r="I173">
         <v>2023</v>
@@ -9569,7 +9524,7 @@
         <v>2015</v>
       </c>
       <c r="O173">
-        <v>74.18183183183194</v>
+        <v>74.5</v>
       </c>
     </row>
     <row r="174">
@@ -9598,7 +9553,7 @@
         </is>
       </c>
       <c r="H174">
-        <v>1.491013071895409</v>
+        <v>1.3125</v>
       </c>
       <c r="I174">
         <v>2023</v>
@@ -9623,7 +9578,7 @@
         <v>2015</v>
       </c>
       <c r="O174">
-        <v>17.2929411764706</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="175">
@@ -9652,7 +9607,7 @@
         </is>
       </c>
       <c r="H175">
-        <v>-3.460597784997937</v>
+        <v>-2.354166666666629</v>
       </c>
       <c r="I175">
         <v>2023</v>
@@ -9677,7 +9632,7 @@
         <v>2015</v>
       </c>
       <c r="O175">
-        <v>87.78787878787878</v>
+        <v>88.5</v>
       </c>
     </row>
     <row r="176">
@@ -9706,7 +9661,7 @@
         </is>
       </c>
       <c r="H176">
-        <v>3.762595762217579</v>
+        <v>3.083333333333307</v>
       </c>
       <c r="I176">
         <v>2023</v>
@@ -9731,7 +9686,7 @@
         <v>2015</v>
       </c>
       <c r="O176">
-        <v>72.69110624794848</v>
+        <v>73.10000000000001</v>
       </c>
     </row>
     <row r="177">
@@ -9760,7 +9715,7 @@
         </is>
       </c>
       <c r="H177">
-        <v>-3.616678083405169</v>
+        <v>-2.966666666666647</v>
       </c>
       <c r="I177">
         <v>2023</v>
@@ -9785,7 +9740,7 @@
         <v>2015</v>
       </c>
       <c r="O177">
-        <v>81.43789297658867</v>
+        <v>81.90000000000015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>